<commit_message>
Add data for 2026-09-04
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -19,18 +19,18 @@
     <sheet name="Rogers Park" sheetId="10" r:id="rId10"/>
     <sheet name="Douglas" sheetId="11" r:id="rId11"/>
     <sheet name="Jefferson Park" sheetId="12" r:id="rId12"/>
-    <sheet name="Grand Crossing" sheetId="13" r:id="rId13"/>
-    <sheet name="Chatham" sheetId="14" r:id="rId14"/>
-    <sheet name="Austin" sheetId="15" r:id="rId15"/>
-    <sheet name="Albany Park" sheetId="16" r:id="rId16"/>
-    <sheet name="Grand Boulevard" sheetId="17" r:id="rId17"/>
-    <sheet name="Belmont Cragin" sheetId="18" r:id="rId18"/>
-    <sheet name="West Ridge" sheetId="19" r:id="rId19"/>
-    <sheet name="Loop" sheetId="20" r:id="rId20"/>
-    <sheet name="Lake View" sheetId="21" r:id="rId21"/>
-    <sheet name="South Shore" sheetId="22" r:id="rId22"/>
-    <sheet name="Mount Greenwood" sheetId="23" r:id="rId23"/>
-    <sheet name="Gage Park" sheetId="24" r:id="rId24"/>
+    <sheet name="Chatham" sheetId="13" r:id="rId13"/>
+    <sheet name="Albany Park" sheetId="14" r:id="rId14"/>
+    <sheet name="Grand Boulevard" sheetId="15" r:id="rId15"/>
+    <sheet name="Belmont Cragin" sheetId="16" r:id="rId16"/>
+    <sheet name="West Ridge" sheetId="17" r:id="rId17"/>
+    <sheet name="Loop" sheetId="18" r:id="rId18"/>
+    <sheet name="Lake View" sheetId="19" r:id="rId19"/>
+    <sheet name="Austin" sheetId="20" r:id="rId20"/>
+    <sheet name="South Shore" sheetId="21" r:id="rId21"/>
+    <sheet name="Mount Greenwood" sheetId="22" r:id="rId22"/>
+    <sheet name="Gage Park" sheetId="23" r:id="rId23"/>
+    <sheet name="Grand Crossing" sheetId="24" r:id="rId24"/>
     <sheet name="West Loop" sheetId="25" r:id="rId25"/>
     <sheet name="Rush &amp; Division" sheetId="26" r:id="rId26"/>
     <sheet name="North Lawndale" sheetId="27" r:id="rId27"/>
@@ -50,9 +50,9 @@
     <sheet name="Roseland" sheetId="41" r:id="rId41"/>
     <sheet name="Woodlawn" sheetId="42" r:id="rId42"/>
     <sheet name="Fuller Park" sheetId="43" r:id="rId43"/>
-    <sheet name="O'Hare" sheetId="44" r:id="rId44"/>
-    <sheet name="Little Italy, UIC" sheetId="45" r:id="rId45"/>
-    <sheet name="Hyde Park" sheetId="46" r:id="rId46"/>
+    <sheet name="Little Italy, UIC" sheetId="44" r:id="rId44"/>
+    <sheet name="Hyde Park" sheetId="45" r:id="rId45"/>
+    <sheet name="O'Hare" sheetId="46" r:id="rId46"/>
     <sheet name="Bucktown" sheetId="47" r:id="rId47"/>
     <sheet name="Calumet Heights" sheetId="48" r:id="rId48"/>
     <sheet name="Edgewater" sheetId="49" r:id="rId49"/>
@@ -2146,41 +2146,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2188,56 +2185,56 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
         <v>8</v>
       </c>
-      <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
-        <v>9</v>
-      </c>
       <c r="H3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L3">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -2245,36 +2242,30 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
+      <c r="J7">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2282,40 +2273,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D8">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G8">
         <v>15</v>
       </c>
       <c r="H8">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I8">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J8">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="K8">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2323,40 +2314,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C9">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E9">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F9">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G9">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H9">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I9">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="J9">
         <v>20</v>
       </c>
       <c r="K9">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="L9">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="M9">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2364,40 +2355,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="C10">
-        <v>106</v>
+        <v>57</v>
       </c>
       <c r="D10">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E10">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="F10">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G10">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H10">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="I10">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="J10">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="K10">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="L10">
-        <v>98</v>
+        <v>40</v>
       </c>
       <c r="M10">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2407,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -2470,38 +2461,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2509,210 +2491,153 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>7</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
       <c r="G3">
-        <v>8</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
       <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="M5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>17</v>
-      </c>
-      <c r="E8">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>19</v>
-      </c>
-      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="K7">
         <v>15</v>
       </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>15</v>
-      </c>
-      <c r="J8">
-        <v>12</v>
-      </c>
-      <c r="K8">
-        <v>18</v>
-      </c>
-      <c r="L8">
-        <v>19</v>
-      </c>
-      <c r="M8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>43</v>
-      </c>
-      <c r="C9">
-        <v>46</v>
-      </c>
-      <c r="D9">
-        <v>32</v>
-      </c>
-      <c r="E9">
-        <v>30</v>
-      </c>
-      <c r="F9">
-        <v>34</v>
-      </c>
-      <c r="G9">
-        <v>15</v>
-      </c>
-      <c r="H9">
-        <v>17</v>
-      </c>
-      <c r="I9">
-        <v>20</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>20</v>
-      </c>
-      <c r="L9">
-        <v>13</v>
-      </c>
-      <c r="M9">
+      <c r="L7">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>51</v>
-      </c>
-      <c r="C10">
-        <v>57</v>
-      </c>
-      <c r="D10">
-        <v>62</v>
-      </c>
-      <c r="E10">
-        <v>48</v>
-      </c>
-      <c r="F10">
-        <v>60</v>
-      </c>
-      <c r="G10">
-        <v>40</v>
-      </c>
-      <c r="H10">
-        <v>31</v>
-      </c>
-      <c r="I10">
-        <v>44</v>
-      </c>
-      <c r="J10">
-        <v>43</v>
-      </c>
-      <c r="K10">
-        <v>57</v>
-      </c>
-      <c r="L10">
-        <v>40</v>
-      </c>
-      <c r="M10">
-        <v>17</v>
+      <c r="M7">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2722,10 +2647,10 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -2785,41 +2710,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2827,210 +2740,162 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>7</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
+        <v>6</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
         <v>6</v>
       </c>
-      <c r="K6">
-        <v>1</v>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>29</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>19</v>
+      </c>
+      <c r="G7">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
       </c>
       <c r="L7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>23</v>
-      </c>
-      <c r="C8">
-        <v>31</v>
-      </c>
-      <c r="D8">
-        <v>22</v>
-      </c>
-      <c r="E8">
-        <v>44</v>
-      </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>24</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="M8">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>46</v>
-      </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>73</v>
-      </c>
-      <c r="F9">
-        <v>114</v>
-      </c>
-      <c r="G9">
-        <v>58</v>
-      </c>
-      <c r="H9">
-        <v>41</v>
-      </c>
-      <c r="I9">
-        <v>44</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>25</v>
-      </c>
-      <c r="L9">
-        <v>27</v>
-      </c>
-      <c r="M9">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>78</v>
-      </c>
-      <c r="C10">
-        <v>99</v>
-      </c>
-      <c r="D10">
-        <v>65</v>
-      </c>
-      <c r="E10">
-        <v>130</v>
-      </c>
-      <c r="F10">
-        <v>167</v>
-      </c>
-      <c r="G10">
-        <v>92</v>
-      </c>
-      <c r="H10">
-        <v>104</v>
-      </c>
-      <c r="I10">
-        <v>89</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>71</v>
-      </c>
-      <c r="L10">
-        <v>61</v>
-      </c>
-      <c r="M10">
-        <v>50</v>
+      <c r="M7">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3106,25 +2971,7 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
       <c r="J2">
-        <v>4</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -3132,25 +2979,16 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
+      <c r="E3">
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -3158,13 +2996,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -3173,28 +3005,22 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -3205,40 +3031,40 @@
         <v>9</v>
       </c>
       <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
         <v>8</v>
       </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
       <c r="F6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3246,40 +3072,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="K7">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3288,474 +3114,6 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>4</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>15</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
-      </c>
-      <c r="K6">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>29</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>16</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
-      <c r="J7">
-        <v>20</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>16</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>7</v>
-      </c>
-      <c r="E7">
-        <v>11</v>
-      </c>
-      <c r="F7">
-        <v>7</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <v>9</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>3</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3926,6 +3284,656 @@
       </c>
       <c r="L8">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>13</v>
+      </c>
+      <c r="I2">
+        <v>14</v>
+      </c>
+      <c r="J2">
+        <v>22</v>
+      </c>
+      <c r="K2">
+        <v>15</v>
+      </c>
+      <c r="L2">
+        <v>15</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <v>18</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>26</v>
+      </c>
+      <c r="H3">
+        <v>23</v>
+      </c>
+      <c r="I3">
+        <v>32</v>
+      </c>
+      <c r="J3">
+        <v>40</v>
+      </c>
+      <c r="K3">
+        <v>26</v>
+      </c>
+      <c r="L3">
+        <v>34</v>
+      </c>
+      <c r="M3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>44</v>
+      </c>
+      <c r="D8">
+        <v>49</v>
+      </c>
+      <c r="E8">
+        <v>67</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>57</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>64</v>
+      </c>
+      <c r="K8">
+        <v>48</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>233</v>
+      </c>
+      <c r="C9">
+        <v>354</v>
+      </c>
+      <c r="D9">
+        <v>538</v>
+      </c>
+      <c r="E9">
+        <v>705</v>
+      </c>
+      <c r="F9">
+        <v>568</v>
+      </c>
+      <c r="G9">
+        <v>168</v>
+      </c>
+      <c r="H9">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>194</v>
+      </c>
+      <c r="J9">
+        <v>122</v>
+      </c>
+      <c r="K9">
+        <v>114</v>
+      </c>
+      <c r="L9">
+        <v>95</v>
+      </c>
+      <c r="M9">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>282</v>
+      </c>
+      <c r="C10">
+        <v>416</v>
+      </c>
+      <c r="D10">
+        <v>617</v>
+      </c>
+      <c r="E10">
+        <v>797</v>
+      </c>
+      <c r="F10">
+        <v>660</v>
+      </c>
+      <c r="G10">
+        <v>257</v>
+      </c>
+      <c r="H10">
+        <v>236</v>
+      </c>
+      <c r="I10">
+        <v>324</v>
+      </c>
+      <c r="J10">
+        <v>255</v>
+      </c>
+      <c r="K10">
+        <v>207</v>
+      </c>
+      <c r="L10">
+        <v>196</v>
+      </c>
+      <c r="M10">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>11</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>17</v>
+      </c>
+      <c r="I6">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>58</v>
+      </c>
+      <c r="C7">
+        <v>53</v>
+      </c>
+      <c r="D7">
+        <v>43</v>
+      </c>
+      <c r="E7">
+        <v>56</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>33</v>
+      </c>
+      <c r="H7">
+        <v>23</v>
+      </c>
+      <c r="I7">
+        <v>26</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>19</v>
+      </c>
+      <c r="M7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>60</v>
+      </c>
+      <c r="C8">
+        <v>76</v>
+      </c>
+      <c r="D8">
+        <v>57</v>
+      </c>
+      <c r="E8">
+        <v>74</v>
+      </c>
+      <c r="F8">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>52</v>
+      </c>
+      <c r="H8">
+        <v>51</v>
+      </c>
+      <c r="I8">
+        <v>52</v>
+      </c>
+      <c r="J8">
+        <v>43</v>
+      </c>
+      <c r="K8">
+        <v>41</v>
+      </c>
+      <c r="L8">
+        <v>39</v>
+      </c>
+      <c r="M8">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -7892,40 +7900,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>13</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>22</v>
-      </c>
       <c r="K2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -7933,59 +7941,47 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>14</v>
       </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>32</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
-      </c>
-      <c r="K3">
-        <v>26</v>
-      </c>
-      <c r="L3">
-        <v>34</v>
-      </c>
       <c r="M3">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
@@ -7993,23 +7989,14 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -8017,30 +8004,15 @@
       <c r="K5">
         <v>2</v>
       </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
       <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+      <c r="K6">
         <v>1</v>
       </c>
     </row>
@@ -8048,7 +8020,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>1</v>
       </c>
     </row>
@@ -8057,40 +8029,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
         <v>44</v>
       </c>
-      <c r="D8">
-        <v>49</v>
-      </c>
-      <c r="E8">
-        <v>67</v>
-      </c>
       <c r="F8">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G8">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="I8">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="J8">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="K8">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -8098,40 +8070,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>233</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>354</v>
+        <v>59</v>
       </c>
       <c r="D9">
-        <v>538</v>
+        <v>33</v>
       </c>
       <c r="E9">
-        <v>705</v>
+        <v>73</v>
       </c>
       <c r="F9">
-        <v>568</v>
+        <v>114</v>
       </c>
       <c r="G9">
-        <v>168</v>
+        <v>58</v>
       </c>
       <c r="H9">
-        <v>116</v>
+        <v>41</v>
       </c>
       <c r="I9">
-        <v>194</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="K9">
-        <v>114</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8139,40 +8111,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>282</v>
+        <v>78</v>
       </c>
       <c r="C10">
-        <v>416</v>
+        <v>99</v>
       </c>
       <c r="D10">
-        <v>617</v>
+        <v>65</v>
       </c>
       <c r="E10">
-        <v>797</v>
+        <v>130</v>
       </c>
       <c r="F10">
-        <v>660</v>
+        <v>167</v>
       </c>
       <c r="G10">
-        <v>257</v>
+        <v>92</v>
       </c>
       <c r="H10">
-        <v>236</v>
+        <v>104</v>
       </c>
       <c r="I10">
-        <v>324</v>
+        <v>89</v>
       </c>
       <c r="J10">
-        <v>255</v>
+        <v>67</v>
       </c>
       <c r="K10">
-        <v>207</v>
+        <v>71</v>
       </c>
       <c r="L10">
-        <v>196</v>
+        <v>61</v>
       </c>
       <c r="M10">
-        <v>88</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -8181,302 +8153,6 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>12</v>
-      </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>17</v>
-      </c>
-      <c r="I6">
-        <v>20</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>10</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>58</v>
-      </c>
-      <c r="C7">
-        <v>53</v>
-      </c>
-      <c r="D7">
-        <v>43</v>
-      </c>
-      <c r="E7">
-        <v>56</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>33</v>
-      </c>
-      <c r="H7">
-        <v>23</v>
-      </c>
-      <c r="I7">
-        <v>26</v>
-      </c>
-      <c r="J7">
-        <v>27</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>19</v>
-      </c>
-      <c r="M7">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>60</v>
-      </c>
-      <c r="C8">
-        <v>76</v>
-      </c>
-      <c r="D8">
-        <v>57</v>
-      </c>
-      <c r="E8">
-        <v>74</v>
-      </c>
-      <c r="F8">
-        <v>71</v>
-      </c>
-      <c r="G8">
-        <v>52</v>
-      </c>
-      <c r="H8">
-        <v>51</v>
-      </c>
-      <c r="I8">
-        <v>52</v>
-      </c>
-      <c r="J8">
-        <v>43</v>
-      </c>
-      <c r="K8">
-        <v>41</v>
-      </c>
-      <c r="L8">
-        <v>39</v>
-      </c>
-      <c r="M8">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8747,7 +8423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8810,7 +8486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9077,6 +8753,330 @@
       </c>
       <c r="M9">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>7</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>19</v>
+      </c>
+      <c r="G3">
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
+      </c>
+      <c r="L3">
+        <v>13</v>
+      </c>
+      <c r="M3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>21</v>
+      </c>
+      <c r="E8">
+        <v>22</v>
+      </c>
+      <c r="F8">
+        <v>27</v>
+      </c>
+      <c r="G8">
+        <v>15</v>
+      </c>
+      <c r="H8">
+        <v>25</v>
+      </c>
+      <c r="I8">
+        <v>21</v>
+      </c>
+      <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>49</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>45</v>
+      </c>
+      <c r="C9">
+        <v>64</v>
+      </c>
+      <c r="D9">
+        <v>46</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9">
+        <v>38</v>
+      </c>
+      <c r="G9">
+        <v>19</v>
+      </c>
+      <c r="H9">
+        <v>27</v>
+      </c>
+      <c r="I9">
+        <v>37</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>35</v>
+      </c>
+      <c r="L9">
+        <v>35</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>77</v>
+      </c>
+      <c r="C10">
+        <v>106</v>
+      </c>
+      <c r="D10">
+        <v>82</v>
+      </c>
+      <c r="E10">
+        <v>88</v>
+      </c>
+      <c r="F10">
+        <v>91</v>
+      </c>
+      <c r="G10">
+        <v>47</v>
+      </c>
+      <c r="H10">
+        <v>66</v>
+      </c>
+      <c r="I10">
+        <v>77</v>
+      </c>
+      <c r="J10">
+        <v>67</v>
+      </c>
+      <c r="K10">
+        <v>110</v>
+      </c>
+      <c r="L10">
+        <v>98</v>
+      </c>
+      <c r="M10">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -14580,257 +14580,6 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>47</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>22</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -15108,7 +14857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15324,6 +15073,257 @@
       </c>
       <c r="M6">
         <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>41</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8">
+        <v>47</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>22</v>
+      </c>
+      <c r="L8">
+        <v>21</v>
+      </c>
+      <c r="M8">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-05
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -19,18 +19,18 @@
     <sheet name="Rogers Park" sheetId="10" r:id="rId10"/>
     <sheet name="Douglas" sheetId="11" r:id="rId11"/>
     <sheet name="Jefferson Park" sheetId="12" r:id="rId12"/>
-    <sheet name="Grand Crossing" sheetId="13" r:id="rId13"/>
-    <sheet name="Chatham" sheetId="14" r:id="rId14"/>
-    <sheet name="Austin" sheetId="15" r:id="rId15"/>
-    <sheet name="Albany Park" sheetId="16" r:id="rId16"/>
-    <sheet name="Grand Boulevard" sheetId="17" r:id="rId17"/>
-    <sheet name="Belmont Cragin" sheetId="18" r:id="rId18"/>
-    <sheet name="West Ridge" sheetId="19" r:id="rId19"/>
-    <sheet name="Loop" sheetId="20" r:id="rId20"/>
-    <sheet name="Lake View" sheetId="21" r:id="rId21"/>
-    <sheet name="South Shore" sheetId="22" r:id="rId22"/>
-    <sheet name="Mount Greenwood" sheetId="23" r:id="rId23"/>
-    <sheet name="Gage Park" sheetId="24" r:id="rId24"/>
+    <sheet name="Chatham" sheetId="13" r:id="rId13"/>
+    <sheet name="Albany Park" sheetId="14" r:id="rId14"/>
+    <sheet name="Grand Boulevard" sheetId="15" r:id="rId15"/>
+    <sheet name="Belmont Cragin" sheetId="16" r:id="rId16"/>
+    <sheet name="West Ridge" sheetId="17" r:id="rId17"/>
+    <sheet name="Loop" sheetId="18" r:id="rId18"/>
+    <sheet name="Lake View" sheetId="19" r:id="rId19"/>
+    <sheet name="Austin" sheetId="20" r:id="rId20"/>
+    <sheet name="South Shore" sheetId="21" r:id="rId21"/>
+    <sheet name="Mount Greenwood" sheetId="22" r:id="rId22"/>
+    <sheet name="Gage Park" sheetId="23" r:id="rId23"/>
+    <sheet name="Grand Crossing" sheetId="24" r:id="rId24"/>
     <sheet name="West Loop" sheetId="25" r:id="rId25"/>
     <sheet name="Rush &amp; Division" sheetId="26" r:id="rId26"/>
     <sheet name="North Lawndale" sheetId="27" r:id="rId27"/>
@@ -50,9 +50,9 @@
     <sheet name="Roseland" sheetId="41" r:id="rId41"/>
     <sheet name="Woodlawn" sheetId="42" r:id="rId42"/>
     <sheet name="Fuller Park" sheetId="43" r:id="rId43"/>
-    <sheet name="O'Hare" sheetId="44" r:id="rId44"/>
-    <sheet name="Little Italy, UIC" sheetId="45" r:id="rId45"/>
-    <sheet name="Hyde Park" sheetId="46" r:id="rId46"/>
+    <sheet name="Little Italy, UIC" sheetId="44" r:id="rId44"/>
+    <sheet name="Hyde Park" sheetId="45" r:id="rId45"/>
+    <sheet name="O'Hare" sheetId="46" r:id="rId46"/>
     <sheet name="Bucktown" sheetId="47" r:id="rId47"/>
     <sheet name="Calumet Heights" sheetId="48" r:id="rId48"/>
     <sheet name="Edgewater" sheetId="49" r:id="rId49"/>
@@ -2146,41 +2146,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2188,56 +2185,56 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
         <v>8</v>
       </c>
-      <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
-        <v>9</v>
-      </c>
       <c r="H3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L3">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -2245,36 +2242,30 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
+      <c r="J7">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2282,40 +2273,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D8">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G8">
         <v>15</v>
       </c>
       <c r="H8">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I8">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J8">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="K8">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2323,40 +2314,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C9">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E9">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F9">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G9">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H9">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I9">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="J9">
         <v>20</v>
       </c>
       <c r="K9">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="L9">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="M9">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2364,40 +2355,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="C10">
-        <v>106</v>
+        <v>57</v>
       </c>
       <c r="D10">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E10">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="F10">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="G10">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H10">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="I10">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="J10">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="K10">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="L10">
-        <v>98</v>
+        <v>40</v>
       </c>
       <c r="M10">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2407,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -2470,38 +2461,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2509,210 +2491,153 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>7</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
       <c r="G3">
-        <v>8</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
       <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="M5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>17</v>
-      </c>
-      <c r="E8">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>19</v>
-      </c>
-      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="K7">
         <v>15</v>
       </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>15</v>
-      </c>
-      <c r="J8">
-        <v>12</v>
-      </c>
-      <c r="K8">
-        <v>18</v>
-      </c>
-      <c r="L8">
-        <v>19</v>
-      </c>
-      <c r="M8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>43</v>
-      </c>
-      <c r="C9">
-        <v>46</v>
-      </c>
-      <c r="D9">
-        <v>32</v>
-      </c>
-      <c r="E9">
-        <v>30</v>
-      </c>
-      <c r="F9">
-        <v>34</v>
-      </c>
-      <c r="G9">
-        <v>15</v>
-      </c>
-      <c r="H9">
-        <v>17</v>
-      </c>
-      <c r="I9">
-        <v>20</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>20</v>
-      </c>
-      <c r="L9">
-        <v>13</v>
-      </c>
-      <c r="M9">
+      <c r="L7">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>51</v>
-      </c>
-      <c r="C10">
-        <v>57</v>
-      </c>
-      <c r="D10">
-        <v>62</v>
-      </c>
-      <c r="E10">
-        <v>48</v>
-      </c>
-      <c r="F10">
-        <v>60</v>
-      </c>
-      <c r="G10">
-        <v>40</v>
-      </c>
-      <c r="H10">
-        <v>31</v>
-      </c>
-      <c r="I10">
-        <v>44</v>
-      </c>
-      <c r="J10">
-        <v>43</v>
-      </c>
-      <c r="K10">
-        <v>57</v>
-      </c>
-      <c r="L10">
-        <v>40</v>
-      </c>
-      <c r="M10">
-        <v>17</v>
+      <c r="M7">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2722,10 +2647,10 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -2785,41 +2710,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2827,210 +2740,162 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>7</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
+        <v>6</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
         <v>6</v>
       </c>
-      <c r="K6">
-        <v>1</v>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>29</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>19</v>
+      </c>
+      <c r="G7">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
       </c>
       <c r="L7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>23</v>
-      </c>
-      <c r="C8">
-        <v>31</v>
-      </c>
-      <c r="D8">
-        <v>22</v>
-      </c>
-      <c r="E8">
-        <v>44</v>
-      </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>24</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="M8">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>46</v>
-      </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>73</v>
-      </c>
-      <c r="F9">
-        <v>114</v>
-      </c>
-      <c r="G9">
-        <v>58</v>
-      </c>
-      <c r="H9">
-        <v>41</v>
-      </c>
-      <c r="I9">
-        <v>44</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>25</v>
-      </c>
-      <c r="L9">
-        <v>27</v>
-      </c>
-      <c r="M9">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>78</v>
-      </c>
-      <c r="C10">
-        <v>99</v>
-      </c>
-      <c r="D10">
-        <v>65</v>
-      </c>
-      <c r="E10">
-        <v>130</v>
-      </c>
-      <c r="F10">
-        <v>167</v>
-      </c>
-      <c r="G10">
-        <v>92</v>
-      </c>
-      <c r="H10">
-        <v>104</v>
-      </c>
-      <c r="I10">
-        <v>89</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>71</v>
-      </c>
-      <c r="L10">
-        <v>61</v>
-      </c>
-      <c r="M10">
-        <v>50</v>
+      <c r="M7">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3106,25 +2971,7 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
       <c r="J2">
-        <v>4</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -3132,25 +2979,16 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
+      <c r="E3">
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -3158,13 +2996,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -3173,28 +3005,22 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -3205,40 +3031,40 @@
         <v>9</v>
       </c>
       <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
         <v>8</v>
       </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
       <c r="F6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3246,40 +3072,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="K7">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3288,474 +3114,6 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>4</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>15</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
-      </c>
-      <c r="K6">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>29</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>16</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
-      <c r="J7">
-        <v>20</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>16</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>7</v>
-      </c>
-      <c r="E7">
-        <v>11</v>
-      </c>
-      <c r="F7">
-        <v>7</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <v>9</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>3</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3926,6 +3284,656 @@
       </c>
       <c r="L8">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>13</v>
+      </c>
+      <c r="I2">
+        <v>14</v>
+      </c>
+      <c r="J2">
+        <v>22</v>
+      </c>
+      <c r="K2">
+        <v>15</v>
+      </c>
+      <c r="L2">
+        <v>15</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <v>18</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>26</v>
+      </c>
+      <c r="H3">
+        <v>23</v>
+      </c>
+      <c r="I3">
+        <v>32</v>
+      </c>
+      <c r="J3">
+        <v>40</v>
+      </c>
+      <c r="K3">
+        <v>26</v>
+      </c>
+      <c r="L3">
+        <v>34</v>
+      </c>
+      <c r="M3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>44</v>
+      </c>
+      <c r="D8">
+        <v>49</v>
+      </c>
+      <c r="E8">
+        <v>67</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>57</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>64</v>
+      </c>
+      <c r="K8">
+        <v>48</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>233</v>
+      </c>
+      <c r="C9">
+        <v>354</v>
+      </c>
+      <c r="D9">
+        <v>538</v>
+      </c>
+      <c r="E9">
+        <v>705</v>
+      </c>
+      <c r="F9">
+        <v>568</v>
+      </c>
+      <c r="G9">
+        <v>168</v>
+      </c>
+      <c r="H9">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>194</v>
+      </c>
+      <c r="J9">
+        <v>122</v>
+      </c>
+      <c r="K9">
+        <v>114</v>
+      </c>
+      <c r="L9">
+        <v>95</v>
+      </c>
+      <c r="M9">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>282</v>
+      </c>
+      <c r="C10">
+        <v>416</v>
+      </c>
+      <c r="D10">
+        <v>617</v>
+      </c>
+      <c r="E10">
+        <v>797</v>
+      </c>
+      <c r="F10">
+        <v>660</v>
+      </c>
+      <c r="G10">
+        <v>257</v>
+      </c>
+      <c r="H10">
+        <v>236</v>
+      </c>
+      <c r="I10">
+        <v>324</v>
+      </c>
+      <c r="J10">
+        <v>255</v>
+      </c>
+      <c r="K10">
+        <v>207</v>
+      </c>
+      <c r="L10">
+        <v>196</v>
+      </c>
+      <c r="M10">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>11</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>17</v>
+      </c>
+      <c r="I6">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>58</v>
+      </c>
+      <c r="C7">
+        <v>53</v>
+      </c>
+      <c r="D7">
+        <v>43</v>
+      </c>
+      <c r="E7">
+        <v>56</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>33</v>
+      </c>
+      <c r="H7">
+        <v>23</v>
+      </c>
+      <c r="I7">
+        <v>26</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>19</v>
+      </c>
+      <c r="M7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>60</v>
+      </c>
+      <c r="C8">
+        <v>76</v>
+      </c>
+      <c r="D8">
+        <v>57</v>
+      </c>
+      <c r="E8">
+        <v>74</v>
+      </c>
+      <c r="F8">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>52</v>
+      </c>
+      <c r="H8">
+        <v>51</v>
+      </c>
+      <c r="I8">
+        <v>52</v>
+      </c>
+      <c r="J8">
+        <v>43</v>
+      </c>
+      <c r="K8">
+        <v>41</v>
+      </c>
+      <c r="L8">
+        <v>39</v>
+      </c>
+      <c r="M8">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -7892,40 +7900,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>13</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>22</v>
-      </c>
       <c r="K2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -7933,59 +7941,47 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>14</v>
       </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>32</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
-      </c>
-      <c r="K3">
-        <v>26</v>
-      </c>
-      <c r="L3">
-        <v>34</v>
-      </c>
       <c r="M3">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
@@ -7993,23 +7989,14 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -8017,30 +8004,15 @@
       <c r="K5">
         <v>2</v>
       </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
       <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+      <c r="K6">
         <v>1</v>
       </c>
     </row>
@@ -8048,7 +8020,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>1</v>
       </c>
     </row>
@@ -8057,40 +8029,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
         <v>44</v>
       </c>
-      <c r="D8">
-        <v>49</v>
-      </c>
-      <c r="E8">
-        <v>67</v>
-      </c>
       <c r="F8">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G8">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="I8">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="J8">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="K8">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="M8">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -8098,40 +8070,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>233</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>354</v>
+        <v>59</v>
       </c>
       <c r="D9">
-        <v>538</v>
+        <v>33</v>
       </c>
       <c r="E9">
-        <v>705</v>
+        <v>73</v>
       </c>
       <c r="F9">
-        <v>568</v>
+        <v>114</v>
       </c>
       <c r="G9">
-        <v>168</v>
+        <v>58</v>
       </c>
       <c r="H9">
-        <v>116</v>
+        <v>41</v>
       </c>
       <c r="I9">
-        <v>194</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="K9">
-        <v>114</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8139,40 +8111,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>282</v>
+        <v>78</v>
       </c>
       <c r="C10">
-        <v>416</v>
+        <v>99</v>
       </c>
       <c r="D10">
-        <v>617</v>
+        <v>65</v>
       </c>
       <c r="E10">
-        <v>797</v>
+        <v>130</v>
       </c>
       <c r="F10">
-        <v>660</v>
+        <v>167</v>
       </c>
       <c r="G10">
-        <v>257</v>
+        <v>92</v>
       </c>
       <c r="H10">
-        <v>236</v>
+        <v>104</v>
       </c>
       <c r="I10">
-        <v>324</v>
+        <v>89</v>
       </c>
       <c r="J10">
-        <v>255</v>
+        <v>67</v>
       </c>
       <c r="K10">
-        <v>207</v>
+        <v>71</v>
       </c>
       <c r="L10">
-        <v>196</v>
+        <v>61</v>
       </c>
       <c r="M10">
-        <v>89</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -8181,302 +8153,6 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>12</v>
-      </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>17</v>
-      </c>
-      <c r="I6">
-        <v>20</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>10</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>58</v>
-      </c>
-      <c r="C7">
-        <v>53</v>
-      </c>
-      <c r="D7">
-        <v>43</v>
-      </c>
-      <c r="E7">
-        <v>56</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>33</v>
-      </c>
-      <c r="H7">
-        <v>23</v>
-      </c>
-      <c r="I7">
-        <v>26</v>
-      </c>
-      <c r="J7">
-        <v>27</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>19</v>
-      </c>
-      <c r="M7">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>60</v>
-      </c>
-      <c r="C8">
-        <v>76</v>
-      </c>
-      <c r="D8">
-        <v>57</v>
-      </c>
-      <c r="E8">
-        <v>74</v>
-      </c>
-      <c r="F8">
-        <v>71</v>
-      </c>
-      <c r="G8">
-        <v>52</v>
-      </c>
-      <c r="H8">
-        <v>51</v>
-      </c>
-      <c r="I8">
-        <v>52</v>
-      </c>
-      <c r="J8">
-        <v>43</v>
-      </c>
-      <c r="K8">
-        <v>41</v>
-      </c>
-      <c r="L8">
-        <v>39</v>
-      </c>
-      <c r="M8">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8747,7 +8423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8810,7 +8486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9077,6 +8753,330 @@
       </c>
       <c r="M9">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>7</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>19</v>
+      </c>
+      <c r="G3">
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
+      </c>
+      <c r="L3">
+        <v>13</v>
+      </c>
+      <c r="M3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>21</v>
+      </c>
+      <c r="E8">
+        <v>22</v>
+      </c>
+      <c r="F8">
+        <v>27</v>
+      </c>
+      <c r="G8">
+        <v>15</v>
+      </c>
+      <c r="H8">
+        <v>25</v>
+      </c>
+      <c r="I8">
+        <v>21</v>
+      </c>
+      <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>49</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>45</v>
+      </c>
+      <c r="C9">
+        <v>64</v>
+      </c>
+      <c r="D9">
+        <v>46</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9">
+        <v>38</v>
+      </c>
+      <c r="G9">
+        <v>19</v>
+      </c>
+      <c r="H9">
+        <v>27</v>
+      </c>
+      <c r="I9">
+        <v>37</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>35</v>
+      </c>
+      <c r="L9">
+        <v>35</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>77</v>
+      </c>
+      <c r="C10">
+        <v>106</v>
+      </c>
+      <c r="D10">
+        <v>82</v>
+      </c>
+      <c r="E10">
+        <v>88</v>
+      </c>
+      <c r="F10">
+        <v>91</v>
+      </c>
+      <c r="G10">
+        <v>47</v>
+      </c>
+      <c r="H10">
+        <v>66</v>
+      </c>
+      <c r="I10">
+        <v>77</v>
+      </c>
+      <c r="J10">
+        <v>67</v>
+      </c>
+      <c r="K10">
+        <v>110</v>
+      </c>
+      <c r="L10">
+        <v>98</v>
+      </c>
+      <c r="M10">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -14580,257 +14580,6 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>47</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>22</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -15108,7 +14857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15324,6 +15073,257 @@
       </c>
       <c r="M6">
         <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>41</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8">
+        <v>47</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>22</v>
+      </c>
+      <c r="L8">
+        <v>21</v>
+      </c>
+      <c r="M8">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-06
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -19,18 +19,18 @@
     <sheet name="Rogers Park" sheetId="10" r:id="rId10"/>
     <sheet name="Douglas" sheetId="11" r:id="rId11"/>
     <sheet name="Jefferson Park" sheetId="12" r:id="rId12"/>
-    <sheet name="Chatham" sheetId="13" r:id="rId13"/>
-    <sheet name="Albany Park" sheetId="14" r:id="rId14"/>
-    <sheet name="Grand Boulevard" sheetId="15" r:id="rId15"/>
-    <sheet name="Belmont Cragin" sheetId="16" r:id="rId16"/>
-    <sheet name="West Ridge" sheetId="17" r:id="rId17"/>
-    <sheet name="Loop" sheetId="18" r:id="rId18"/>
-    <sheet name="Lake View" sheetId="19" r:id="rId19"/>
-    <sheet name="Austin" sheetId="20" r:id="rId20"/>
-    <sheet name="South Shore" sheetId="21" r:id="rId21"/>
-    <sheet name="Mount Greenwood" sheetId="22" r:id="rId22"/>
-    <sheet name="Gage Park" sheetId="23" r:id="rId23"/>
-    <sheet name="Grand Crossing" sheetId="24" r:id="rId24"/>
+    <sheet name="Grand Crossing" sheetId="13" r:id="rId13"/>
+    <sheet name="Chatham" sheetId="14" r:id="rId14"/>
+    <sheet name="Austin" sheetId="15" r:id="rId15"/>
+    <sheet name="Albany Park" sheetId="16" r:id="rId16"/>
+    <sheet name="Grand Boulevard" sheetId="17" r:id="rId17"/>
+    <sheet name="Belmont Cragin" sheetId="18" r:id="rId18"/>
+    <sheet name="West Ridge" sheetId="19" r:id="rId19"/>
+    <sheet name="Loop" sheetId="20" r:id="rId20"/>
+    <sheet name="Lake View" sheetId="21" r:id="rId21"/>
+    <sheet name="South Shore" sheetId="22" r:id="rId22"/>
+    <sheet name="Mount Greenwood" sheetId="23" r:id="rId23"/>
+    <sheet name="Gage Park" sheetId="24" r:id="rId24"/>
     <sheet name="West Loop" sheetId="25" r:id="rId25"/>
     <sheet name="Rush &amp; Division" sheetId="26" r:id="rId26"/>
     <sheet name="North Lawndale" sheetId="27" r:id="rId27"/>
@@ -50,9 +50,9 @@
     <sheet name="Roseland" sheetId="41" r:id="rId41"/>
     <sheet name="Woodlawn" sheetId="42" r:id="rId42"/>
     <sheet name="Fuller Park" sheetId="43" r:id="rId43"/>
-    <sheet name="Little Italy, UIC" sheetId="44" r:id="rId44"/>
-    <sheet name="Hyde Park" sheetId="45" r:id="rId45"/>
-    <sheet name="O'Hare" sheetId="46" r:id="rId46"/>
+    <sheet name="O'Hare" sheetId="44" r:id="rId44"/>
+    <sheet name="Little Italy, UIC" sheetId="45" r:id="rId45"/>
+    <sheet name="Hyde Park" sheetId="46" r:id="rId46"/>
     <sheet name="Bucktown" sheetId="47" r:id="rId47"/>
     <sheet name="Calumet Heights" sheetId="48" r:id="rId48"/>
     <sheet name="Edgewater" sheetId="49" r:id="rId49"/>
@@ -905,7 +905,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1156,7 +1156,7 @@
         <v>467</v>
       </c>
       <c r="M9">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>793</v>
+        <v>796</v>
       </c>
     </row>
   </sheetData>
@@ -2146,38 +2146,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2185,56 +2188,56 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>19</v>
+      </c>
+      <c r="G3">
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
+      </c>
+      <c r="L3">
+        <v>13</v>
+      </c>
+      <c r="M3">
         <v>7</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3">
-        <v>8</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
-      </c>
-      <c r="L3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4">
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -2242,30 +2245,36 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="M6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="J7">
-        <v>2</v>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2273,40 +2282,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="D8">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F8">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G8">
         <v>15</v>
       </c>
       <c r="H8">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I8">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>49</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
         <v>12</v>
-      </c>
-      <c r="K8">
-        <v>18</v>
-      </c>
-      <c r="L8">
-        <v>19</v>
-      </c>
-      <c r="M8">
-        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2314,40 +2323,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C9">
+        <v>64</v>
+      </c>
+      <c r="D9">
         <v>46</v>
       </c>
-      <c r="D9">
-        <v>32</v>
-      </c>
       <c r="E9">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F9">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G9">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="I9">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="J9">
         <v>20</v>
       </c>
       <c r="K9">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="L9">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="M9">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2355,40 +2364,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="C10">
-        <v>57</v>
+        <v>106</v>
       </c>
       <c r="D10">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="E10">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="F10">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G10">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="H10">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="I10">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="J10">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="K10">
-        <v>57</v>
+        <v>110</v>
       </c>
       <c r="L10">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="M10">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2398,7 +2407,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -2461,29 +2470,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2491,153 +2509,210 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
       <c r="G3">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>10</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
       <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
-      <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>17</v>
+      </c>
+      <c r="E8">
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <v>19</v>
+      </c>
+      <c r="G8">
+        <v>15</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>15</v>
+      </c>
+      <c r="J8">
+        <v>12</v>
+      </c>
+      <c r="K8">
+        <v>18</v>
+      </c>
+      <c r="L8">
+        <v>19</v>
+      </c>
+      <c r="M8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>43</v>
+      </c>
+      <c r="C9">
+        <v>46</v>
+      </c>
+      <c r="D9">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9">
+        <v>34</v>
+      </c>
+      <c r="G9">
+        <v>15</v>
+      </c>
+      <c r="H9">
+        <v>17</v>
+      </c>
+      <c r="I9">
+        <v>20</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>20</v>
+      </c>
+      <c r="L9">
+        <v>13</v>
+      </c>
+      <c r="M9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>15</v>
-      </c>
-      <c r="D7">
-        <v>13</v>
-      </c>
-      <c r="E7">
-        <v>13</v>
-      </c>
-      <c r="F7">
-        <v>10</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>14</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
-      <c r="M7">
-        <v>5</v>
+      <c r="B10">
+        <v>51</v>
+      </c>
+      <c r="C10">
+        <v>57</v>
+      </c>
+      <c r="D10">
+        <v>62</v>
+      </c>
+      <c r="E10">
+        <v>48</v>
+      </c>
+      <c r="F10">
+        <v>60</v>
+      </c>
+      <c r="G10">
+        <v>40</v>
+      </c>
+      <c r="H10">
+        <v>31</v>
+      </c>
+      <c r="I10">
+        <v>44</v>
+      </c>
+      <c r="J10">
+        <v>43</v>
+      </c>
+      <c r="K10">
+        <v>57</v>
+      </c>
+      <c r="L10">
+        <v>40</v>
+      </c>
+      <c r="M10">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2647,10 +2722,10 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -2710,29 +2785,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2740,162 +2827,210 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>15</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K6">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
+        <v>44</v>
+      </c>
+      <c r="F8">
+        <v>38</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8">
+        <v>50</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>24</v>
+      </c>
+      <c r="L8">
+        <v>14</v>
+      </c>
+      <c r="M8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="E9">
+        <v>73</v>
+      </c>
+      <c r="F9">
+        <v>114</v>
+      </c>
+      <c r="G9">
+        <v>58</v>
+      </c>
+      <c r="H9">
+        <v>41</v>
+      </c>
+      <c r="I9">
+        <v>44</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>25</v>
+      </c>
+      <c r="L9">
+        <v>27</v>
+      </c>
+      <c r="M9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>29</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>16</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
-      <c r="J7">
-        <v>20</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>16</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
+      <c r="B10">
+        <v>78</v>
+      </c>
+      <c r="C10">
+        <v>99</v>
+      </c>
+      <c r="D10">
+        <v>65</v>
+      </c>
+      <c r="E10">
+        <v>130</v>
+      </c>
+      <c r="F10">
+        <v>167</v>
+      </c>
+      <c r="G10">
+        <v>92</v>
+      </c>
+      <c r="H10">
+        <v>104</v>
+      </c>
+      <c r="I10">
+        <v>89</v>
+      </c>
+      <c r="J10">
+        <v>67</v>
+      </c>
+      <c r="K10">
+        <v>71</v>
+      </c>
+      <c r="L10">
+        <v>61</v>
+      </c>
+      <c r="M10">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2971,7 +3106,25 @@
       <c r="D2">
         <v>1</v>
       </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
       <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -2979,16 +3132,25 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>2</v>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
       </c>
       <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -2996,7 +3158,13 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
@@ -3005,22 +3173,28 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -3031,40 +3205,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
+      </c>
+      <c r="G6">
         <v>8</v>
       </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3072,40 +3246,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="L7">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3114,6 +3288,477 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>29</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>19</v>
+      </c>
+      <c r="G7">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7">
+        <v>16</v>
+      </c>
+      <c r="M7">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>9</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>9</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3284,656 +3929,6 @@
       </c>
       <c r="L8">
         <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>12</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>8</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>13</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>22</v>
-      </c>
-      <c r="K2">
-        <v>15</v>
-      </c>
-      <c r="L2">
-        <v>15</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>13</v>
-      </c>
-      <c r="D3">
-        <v>17</v>
-      </c>
-      <c r="E3">
-        <v>18</v>
-      </c>
-      <c r="F3">
-        <v>14</v>
-      </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>32</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
-      </c>
-      <c r="K3">
-        <v>26</v>
-      </c>
-      <c r="L3">
-        <v>34</v>
-      </c>
-      <c r="M3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>30</v>
-      </c>
-      <c r="C8">
-        <v>44</v>
-      </c>
-      <c r="D8">
-        <v>49</v>
-      </c>
-      <c r="E8">
-        <v>67</v>
-      </c>
-      <c r="F8">
-        <v>69</v>
-      </c>
-      <c r="G8">
-        <v>57</v>
-      </c>
-      <c r="H8">
-        <v>80</v>
-      </c>
-      <c r="I8">
-        <v>80</v>
-      </c>
-      <c r="J8">
-        <v>64</v>
-      </c>
-      <c r="K8">
-        <v>48</v>
-      </c>
-      <c r="L8">
-        <v>44</v>
-      </c>
-      <c r="M8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>233</v>
-      </c>
-      <c r="C9">
-        <v>354</v>
-      </c>
-      <c r="D9">
-        <v>538</v>
-      </c>
-      <c r="E9">
-        <v>705</v>
-      </c>
-      <c r="F9">
-        <v>568</v>
-      </c>
-      <c r="G9">
-        <v>168</v>
-      </c>
-      <c r="H9">
-        <v>116</v>
-      </c>
-      <c r="I9">
-        <v>194</v>
-      </c>
-      <c r="J9">
-        <v>122</v>
-      </c>
-      <c r="K9">
-        <v>114</v>
-      </c>
-      <c r="L9">
-        <v>95</v>
-      </c>
-      <c r="M9">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>282</v>
-      </c>
-      <c r="C10">
-        <v>416</v>
-      </c>
-      <c r="D10">
-        <v>617</v>
-      </c>
-      <c r="E10">
-        <v>797</v>
-      </c>
-      <c r="F10">
-        <v>660</v>
-      </c>
-      <c r="G10">
-        <v>257</v>
-      </c>
-      <c r="H10">
-        <v>236</v>
-      </c>
-      <c r="I10">
-        <v>324</v>
-      </c>
-      <c r="J10">
-        <v>255</v>
-      </c>
-      <c r="K10">
-        <v>207</v>
-      </c>
-      <c r="L10">
-        <v>196</v>
-      </c>
-      <c r="M10">
-        <v>89</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>12</v>
-      </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>17</v>
-      </c>
-      <c r="I6">
-        <v>20</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>10</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>58</v>
-      </c>
-      <c r="C7">
-        <v>53</v>
-      </c>
-      <c r="D7">
-        <v>43</v>
-      </c>
-      <c r="E7">
-        <v>56</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>33</v>
-      </c>
-      <c r="H7">
-        <v>23</v>
-      </c>
-      <c r="I7">
-        <v>26</v>
-      </c>
-      <c r="J7">
-        <v>27</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>19</v>
-      </c>
-      <c r="M7">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>60</v>
-      </c>
-      <c r="C8">
-        <v>76</v>
-      </c>
-      <c r="D8">
-        <v>57</v>
-      </c>
-      <c r="E8">
-        <v>74</v>
-      </c>
-      <c r="F8">
-        <v>71</v>
-      </c>
-      <c r="G8">
-        <v>52</v>
-      </c>
-      <c r="H8">
-        <v>51</v>
-      </c>
-      <c r="I8">
-        <v>52</v>
-      </c>
-      <c r="J8">
-        <v>43</v>
-      </c>
-      <c r="K8">
-        <v>41</v>
-      </c>
-      <c r="L8">
-        <v>39</v>
-      </c>
-      <c r="M8">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -4382,7 +4377,7 @@
         <v>3</v>
       </c>
       <c r="M11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6313,7 +6308,7 @@
         <v>4</v>
       </c>
       <c r="M63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -7287,7 +7282,7 @@
         <v>2</v>
       </c>
       <c r="M88">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -7442,7 +7437,7 @@
         <v>26</v>
       </c>
       <c r="M92">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -7644,7 +7639,7 @@
         <v>6</v>
       </c>
       <c r="M97">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -7726,7 +7721,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>793</v>
+        <v>796</v>
       </c>
     </row>
   </sheetData>
@@ -7900,40 +7895,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -7941,47 +7936,59 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I4">
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -7989,14 +7996,23 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>1</v>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -8004,15 +8020,30 @@
       <c r="K5">
         <v>2</v>
       </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
       <c r="M5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K6">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
         <v>1</v>
       </c>
     </row>
@@ -8020,7 +8051,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L7">
+      <c r="K7">
         <v>1</v>
       </c>
     </row>
@@ -8029,40 +8060,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C8">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D8">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="E8">
+        <v>67</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>57</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>64</v>
+      </c>
+      <c r="K8">
+        <v>48</v>
+      </c>
+      <c r="L8">
         <v>44</v>
       </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>24</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
       <c r="M8">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -8070,40 +8101,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>46</v>
+        <v>233</v>
       </c>
       <c r="C9">
-        <v>59</v>
+        <v>354</v>
       </c>
       <c r="D9">
-        <v>33</v>
+        <v>538</v>
       </c>
       <c r="E9">
-        <v>73</v>
+        <v>705</v>
       </c>
       <c r="F9">
+        <v>568</v>
+      </c>
+      <c r="G9">
+        <v>168</v>
+      </c>
+      <c r="H9">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>194</v>
+      </c>
+      <c r="J9">
+        <v>122</v>
+      </c>
+      <c r="K9">
         <v>114</v>
       </c>
-      <c r="G9">
-        <v>58</v>
-      </c>
-      <c r="H9">
-        <v>41</v>
-      </c>
-      <c r="I9">
-        <v>44</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>25</v>
-      </c>
       <c r="L9">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8111,40 +8142,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>78</v>
+        <v>282</v>
       </c>
       <c r="C10">
-        <v>99</v>
+        <v>416</v>
       </c>
       <c r="D10">
-        <v>65</v>
+        <v>617</v>
       </c>
       <c r="E10">
-        <v>130</v>
+        <v>797</v>
       </c>
       <c r="F10">
-        <v>167</v>
+        <v>660</v>
       </c>
       <c r="G10">
-        <v>92</v>
+        <v>257</v>
       </c>
       <c r="H10">
-        <v>104</v>
+        <v>236</v>
       </c>
       <c r="I10">
+        <v>324</v>
+      </c>
+      <c r="J10">
+        <v>255</v>
+      </c>
+      <c r="K10">
+        <v>207</v>
+      </c>
+      <c r="L10">
+        <v>196</v>
+      </c>
+      <c r="M10">
         <v>89</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>71</v>
-      </c>
-      <c r="L10">
-        <v>61</v>
-      </c>
-      <c r="M10">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -8153,6 +8184,302 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>11</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>17</v>
+      </c>
+      <c r="I6">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>58</v>
+      </c>
+      <c r="C7">
+        <v>53</v>
+      </c>
+      <c r="D7">
+        <v>43</v>
+      </c>
+      <c r="E7">
+        <v>56</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>33</v>
+      </c>
+      <c r="H7">
+        <v>23</v>
+      </c>
+      <c r="I7">
+        <v>26</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>19</v>
+      </c>
+      <c r="M7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>60</v>
+      </c>
+      <c r="C8">
+        <v>76</v>
+      </c>
+      <c r="D8">
+        <v>57</v>
+      </c>
+      <c r="E8">
+        <v>74</v>
+      </c>
+      <c r="F8">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>52</v>
+      </c>
+      <c r="H8">
+        <v>51</v>
+      </c>
+      <c r="I8">
+        <v>52</v>
+      </c>
+      <c r="J8">
+        <v>43</v>
+      </c>
+      <c r="K8">
+        <v>41</v>
+      </c>
+      <c r="L8">
+        <v>39</v>
+      </c>
+      <c r="M8">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8423,7 +8750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8486,7 +8813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8753,330 +9080,6 @@
       </c>
       <c r="M9">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>6</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>7</v>
-      </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
-        <v>9</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>17</v>
-      </c>
-      <c r="L3">
-        <v>13</v>
-      </c>
-      <c r="M3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>24</v>
-      </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>21</v>
-      </c>
-      <c r="E8">
-        <v>22</v>
-      </c>
-      <c r="F8">
-        <v>27</v>
-      </c>
-      <c r="G8">
-        <v>15</v>
-      </c>
-      <c r="H8">
-        <v>25</v>
-      </c>
-      <c r="I8">
-        <v>21</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>49</v>
-      </c>
-      <c r="L8">
-        <v>44</v>
-      </c>
-      <c r="M8">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>45</v>
-      </c>
-      <c r="C9">
-        <v>64</v>
-      </c>
-      <c r="D9">
-        <v>46</v>
-      </c>
-      <c r="E9">
-        <v>50</v>
-      </c>
-      <c r="F9">
-        <v>38</v>
-      </c>
-      <c r="G9">
-        <v>19</v>
-      </c>
-      <c r="H9">
-        <v>27</v>
-      </c>
-      <c r="I9">
-        <v>37</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>35</v>
-      </c>
-      <c r="L9">
-        <v>35</v>
-      </c>
-      <c r="M9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>77</v>
-      </c>
-      <c r="C10">
-        <v>106</v>
-      </c>
-      <c r="D10">
-        <v>82</v>
-      </c>
-      <c r="E10">
-        <v>88</v>
-      </c>
-      <c r="F10">
-        <v>91</v>
-      </c>
-      <c r="G10">
-        <v>47</v>
-      </c>
-      <c r="H10">
-        <v>66</v>
-      </c>
-      <c r="I10">
-        <v>77</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>110</v>
-      </c>
-      <c r="L10">
-        <v>98</v>
-      </c>
-      <c r="M10">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -9280,7 +9283,7 @@
         <v>5</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -9362,7 +9365,7 @@
         <v>26</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -11325,6 +11328,9 @@
       <c r="K4">
         <v>2</v>
       </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
@@ -11405,7 +11411,7 @@
         <v>4</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -14156,7 +14162,7 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -14290,7 +14296,7 @@
         <v>6</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -14580,6 +14586,257 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>41</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8">
+        <v>47</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>22</v>
+      </c>
+      <c r="L8">
+        <v>21</v>
+      </c>
+      <c r="M8">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -14857,7 +15114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15073,257 +15330,6 @@
       </c>
       <c r="M6">
         <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>47</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>22</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -19262,7 +19268,7 @@
         <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -19375,7 +19381,7 @@
         <v>2</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-07
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -72,13 +72,13 @@
     <sheet name="Brighton Park" sheetId="63" r:id="rId63"/>
     <sheet name="Lincoln Park" sheetId="64" r:id="rId64"/>
     <sheet name="Printers Row" sheetId="65" r:id="rId65"/>
-    <sheet name="West Pullman" sheetId="66" r:id="rId66"/>
-    <sheet name="West Lawn" sheetId="67" r:id="rId67"/>
-    <sheet name="Little Village" sheetId="68" r:id="rId68"/>
-    <sheet name="Ukrainian Village" sheetId="69" r:id="rId69"/>
-    <sheet name="Archer Heights" sheetId="70" r:id="rId70"/>
-    <sheet name="Montclare" sheetId="71" r:id="rId71"/>
-    <sheet name="Old Town" sheetId="72" r:id="rId72"/>
+    <sheet name="Old Town" sheetId="66" r:id="rId66"/>
+    <sheet name="West Pullman" sheetId="67" r:id="rId67"/>
+    <sheet name="West Lawn" sheetId="68" r:id="rId68"/>
+    <sheet name="Little Village" sheetId="69" r:id="rId69"/>
+    <sheet name="Ukrainian Village" sheetId="70" r:id="rId70"/>
+    <sheet name="Archer Heights" sheetId="71" r:id="rId71"/>
+    <sheet name="Montclare" sheetId="72" r:id="rId72"/>
     <sheet name="Grant Park" sheetId="73" r:id="rId73"/>
     <sheet name="West Elsdon" sheetId="74" r:id="rId74"/>
     <sheet name="East Side" sheetId="75" r:id="rId75"/>
@@ -946,7 +946,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1156,7 +1156,7 @@
         <v>467</v>
       </c>
       <c r="M9">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -2306,7 +2306,7 @@
         <v>19</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2388,7 +2388,7 @@
         <v>40</v>
       </c>
       <c r="M10">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -3599,7 +3599,7 @@
         <v>95</v>
       </c>
       <c r="M9">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3640,7 +3640,7 @@
         <v>196</v>
       </c>
       <c r="M10">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -4265,7 +4265,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4665,7 +4665,7 @@
         <v>40</v>
       </c>
       <c r="M19">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -5957,7 +5957,7 @@
         <v>196</v>
       </c>
       <c r="M53">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -6594,7 +6594,7 @@
         <v>17</v>
       </c>
       <c r="M70">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -7729,7 +7729,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -7977,7 +7977,7 @@
         <v>14</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8147,7 +8147,7 @@
         <v>61</v>
       </c>
       <c r="M10">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -20278,6 +20278,272 @@
 
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>17</v>
+      </c>
+      <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>17</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>17</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>26</v>
+      </c>
+      <c r="D7">
+        <v>44</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>79</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>13</v>
+      </c>
+      <c r="I7">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>9</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>53</v>
+      </c>
+      <c r="E8">
+        <v>76</v>
+      </c>
+      <c r="F8">
+        <v>103</v>
+      </c>
+      <c r="G8">
+        <v>39</v>
+      </c>
+      <c r="H8">
+        <v>30</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>29</v>
+      </c>
+      <c r="K8">
+        <v>33</v>
+      </c>
+      <c r="L8">
+        <v>17</v>
+      </c>
+      <c r="M8">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -20496,7 +20762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -20638,7 +20904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -20874,190 +21140,6 @@
       </c>
       <c r="M7">
         <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>3</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -21383,6 +21465,190 @@
 
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -21543,7 +21809,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -21646,272 +21912,6 @@
       </c>
       <c r="G5">
         <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>4</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>6</v>
-      </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>17</v>
-      </c>
-      <c r="F6">
-        <v>18</v>
-      </c>
-      <c r="G6">
-        <v>12</v>
-      </c>
-      <c r="H6">
-        <v>12</v>
-      </c>
-      <c r="I6">
-        <v>17</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>17</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>26</v>
-      </c>
-      <c r="D7">
-        <v>44</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>79</v>
-      </c>
-      <c r="G7">
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <v>13</v>
-      </c>
-      <c r="I7">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>9</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>27</v>
-      </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>53</v>
-      </c>
-      <c r="E8">
-        <v>76</v>
-      </c>
-      <c r="F8">
-        <v>103</v>
-      </c>
-      <c r="G8">
-        <v>39</v>
-      </c>
-      <c r="H8">
-        <v>30</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>29</v>
-      </c>
-      <c r="K8">
-        <v>33</v>
-      </c>
-      <c r="L8">
-        <v>17</v>
-      </c>
-      <c r="M8">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-08
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -9,10 +9,10 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Austin" sheetId="3" r:id="rId3"/>
-    <sheet name="Loop" sheetId="4" r:id="rId4"/>
-    <sheet name="Old Town" sheetId="5" r:id="rId5"/>
-    <sheet name="Chatham" sheetId="6" r:id="rId6"/>
+    <sheet name="Chatham" sheetId="3" r:id="rId3"/>
+    <sheet name="Austin" sheetId="4" r:id="rId4"/>
+    <sheet name="Loop" sheetId="5" r:id="rId5"/>
+    <sheet name="Old Town" sheetId="6" r:id="rId6"/>
     <sheet name="New City" sheetId="7" r:id="rId7"/>
     <sheet name="Belmont Cragin" sheetId="8" r:id="rId8"/>
     <sheet name="Woodlawn" sheetId="9" r:id="rId9"/>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>800</v>
+        <v>802</v>
       </c>
     </row>
   </sheetData>
@@ -4617,7 +4617,7 @@
         <v>40</v>
       </c>
       <c r="M19">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -5251,7 +5251,7 @@
         <v>98</v>
       </c>
       <c r="M36">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7681,7 +7681,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>800</v>
+        <v>802</v>
       </c>
     </row>
   </sheetData>
@@ -10595,41 +10595,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2">
         <v>8</v>
       </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -10637,47 +10634,47 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>6</v>
       </c>
       <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
         <v>10</v>
       </c>
-      <c r="K3">
-        <v>12</v>
-      </c>
       <c r="L3">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I4">
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
@@ -10688,19 +10685,7 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -10708,7 +10693,13 @@
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K6">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>1</v>
       </c>
     </row>
@@ -10716,8 +10707,14 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L7">
-        <v>1</v>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -10725,40 +10722,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D8">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G8">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H8">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="I8">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="J8">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="K8">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L8">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="M8">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -10766,40 +10763,40 @@
         <v>9</v>
       </c>
       <c r="B9">
+        <v>43</v>
+      </c>
+      <c r="C9">
         <v>46</v>
       </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
       <c r="D9">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="F9">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="G9">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="H9">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="I9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="J9">
         <v>20</v>
       </c>
       <c r="K9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="L9">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -10807,40 +10804,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="C10">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="D10">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E10">
-        <v>130</v>
+        <v>48</v>
       </c>
       <c r="F10">
-        <v>167</v>
+        <v>60</v>
       </c>
       <c r="G10">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="H10">
-        <v>104</v>
+        <v>31</v>
       </c>
       <c r="I10">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="J10">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="K10">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="L10">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="M10">
-        <v>51</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -11848,6 +11845,9 @@
       <c r="L7">
         <v>1</v>
       </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
@@ -11969,7 +11969,7 @@
         <v>98</v>
       </c>
       <c r="M10">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -13481,40 +13481,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>13</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>22</v>
-      </c>
       <c r="K2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13522,59 +13522,47 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>14</v>
       </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>32</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
-      </c>
-      <c r="K3">
-        <v>26</v>
-      </c>
-      <c r="L3">
-        <v>34</v>
-      </c>
       <c r="M3">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
@@ -13582,23 +13570,14 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -13606,30 +13585,15 @@
       <c r="K5">
         <v>2</v>
       </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
       <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+      <c r="K6">
         <v>1</v>
       </c>
     </row>
@@ -13637,7 +13601,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>1</v>
       </c>
     </row>
@@ -13646,40 +13610,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
         <v>44</v>
       </c>
-      <c r="D8">
-        <v>49</v>
-      </c>
-      <c r="E8">
-        <v>67</v>
-      </c>
       <c r="F8">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G8">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="I8">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="J8">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="K8">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="M8">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13687,40 +13651,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>233</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>354</v>
+        <v>59</v>
       </c>
       <c r="D9">
-        <v>538</v>
+        <v>33</v>
       </c>
       <c r="E9">
-        <v>705</v>
+        <v>73</v>
       </c>
       <c r="F9">
-        <v>568</v>
+        <v>114</v>
       </c>
       <c r="G9">
-        <v>168</v>
+        <v>58</v>
       </c>
       <c r="H9">
-        <v>116</v>
+        <v>41</v>
       </c>
       <c r="I9">
-        <v>194</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="K9">
-        <v>114</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13728,40 +13692,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>282</v>
+        <v>78</v>
       </c>
       <c r="C10">
-        <v>416</v>
+        <v>99</v>
       </c>
       <c r="D10">
-        <v>617</v>
+        <v>65</v>
       </c>
       <c r="E10">
-        <v>797</v>
+        <v>130</v>
       </c>
       <c r="F10">
-        <v>660</v>
+        <v>167</v>
       </c>
       <c r="G10">
-        <v>257</v>
+        <v>92</v>
       </c>
       <c r="H10">
-        <v>236</v>
+        <v>104</v>
       </c>
       <c r="I10">
-        <v>324</v>
+        <v>89</v>
       </c>
       <c r="J10">
-        <v>255</v>
+        <v>67</v>
       </c>
       <c r="K10">
-        <v>207</v>
+        <v>71</v>
       </c>
       <c r="L10">
-        <v>196</v>
+        <v>61</v>
       </c>
       <c r="M10">
-        <v>90</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -16239,7 +16203,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -16302,25 +16266,40 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
       <c r="D2">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="I2">
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="L2">
+        <v>15</v>
+      </c>
+      <c r="M2">
         <v>2</v>
       </c>
     </row>
@@ -16329,41 +16308,59 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>3</v>
+        <v>34</v>
+      </c>
+      <c r="M3">
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -16371,131 +16368,186 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>17</v>
-      </c>
-      <c r="F6">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>12</v>
-      </c>
-      <c r="I6">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>26</v>
-      </c>
-      <c r="D7">
-        <v>44</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>79</v>
-      </c>
-      <c r="G7">
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <v>13</v>
-      </c>
-      <c r="I7">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K7">
-        <v>9</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>44</v>
+      </c>
+      <c r="D8">
+        <v>49</v>
+      </c>
+      <c r="E8">
+        <v>67</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>57</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>64</v>
+      </c>
+      <c r="K8">
+        <v>48</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>233</v>
+      </c>
+      <c r="C9">
+        <v>354</v>
+      </c>
+      <c r="D9">
+        <v>538</v>
+      </c>
+      <c r="E9">
+        <v>705</v>
+      </c>
+      <c r="F9">
+        <v>568</v>
+      </c>
+      <c r="G9">
+        <v>168</v>
+      </c>
+      <c r="H9">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>194</v>
+      </c>
+      <c r="J9">
+        <v>122</v>
+      </c>
+      <c r="K9">
+        <v>114</v>
+      </c>
+      <c r="L9">
+        <v>95</v>
+      </c>
+      <c r="M9">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8">
-        <v>27</v>
-      </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>53</v>
-      </c>
-      <c r="E8">
-        <v>76</v>
-      </c>
-      <c r="F8">
-        <v>103</v>
-      </c>
-      <c r="G8">
-        <v>39</v>
-      </c>
-      <c r="H8">
-        <v>30</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>29</v>
-      </c>
-      <c r="K8">
-        <v>33</v>
-      </c>
-      <c r="L8">
-        <v>17</v>
-      </c>
-      <c r="M8">
-        <v>7</v>
+      <c r="B10">
+        <v>282</v>
+      </c>
+      <c r="C10">
+        <v>416</v>
+      </c>
+      <c r="D10">
+        <v>617</v>
+      </c>
+      <c r="E10">
+        <v>797</v>
+      </c>
+      <c r="F10">
+        <v>660</v>
+      </c>
+      <c r="G10">
+        <v>257</v>
+      </c>
+      <c r="H10">
+        <v>236</v>
+      </c>
+      <c r="I10">
+        <v>324</v>
+      </c>
+      <c r="J10">
+        <v>255</v>
+      </c>
+      <c r="K10">
+        <v>207</v>
+      </c>
+      <c r="L10">
+        <v>196</v>
+      </c>
+      <c r="M10">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -18921,7 +18973,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -18984,38 +19036,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>3</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -19023,47 +19063,41 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
         <v>4</v>
       </c>
       <c r="G3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>4</v>
       </c>
       <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
         <v>6</v>
       </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
       <c r="K3">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
@@ -19071,162 +19105,131 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="K5">
+      <c r="J5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>17</v>
+      </c>
+      <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>17</v>
+      </c>
+      <c r="J6">
         <v>6</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
+      <c r="K6">
+        <v>17</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>26</v>
+      </c>
+      <c r="D7">
+        <v>44</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>79</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>13</v>
+      </c>
+      <c r="I7">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>9</v>
+      </c>
+      <c r="L7">
         <v>7</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <v>2</v>
+      <c r="M7">
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C8">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="D8">
+        <v>53</v>
+      </c>
+      <c r="E8">
+        <v>76</v>
+      </c>
+      <c r="F8">
+        <v>103</v>
+      </c>
+      <c r="G8">
+        <v>39</v>
+      </c>
+      <c r="H8">
+        <v>30</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>29</v>
+      </c>
+      <c r="K8">
+        <v>33</v>
+      </c>
+      <c r="L8">
         <v>17</v>
       </c>
-      <c r="E8">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>19</v>
-      </c>
-      <c r="G8">
-        <v>15</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>15</v>
-      </c>
-      <c r="J8">
-        <v>12</v>
-      </c>
-      <c r="K8">
-        <v>18</v>
-      </c>
-      <c r="L8">
-        <v>19</v>
-      </c>
       <c r="M8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>43</v>
-      </c>
-      <c r="C9">
-        <v>46</v>
-      </c>
-      <c r="D9">
-        <v>32</v>
-      </c>
-      <c r="E9">
-        <v>30</v>
-      </c>
-      <c r="F9">
-        <v>34</v>
-      </c>
-      <c r="G9">
-        <v>15</v>
-      </c>
-      <c r="H9">
-        <v>17</v>
-      </c>
-      <c r="I9">
-        <v>20</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>20</v>
-      </c>
-      <c r="L9">
-        <v>13</v>
-      </c>
-      <c r="M9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>51</v>
-      </c>
-      <c r="C10">
-        <v>57</v>
-      </c>
-      <c r="D10">
-        <v>62</v>
-      </c>
-      <c r="E10">
-        <v>48</v>
-      </c>
-      <c r="F10">
-        <v>60</v>
-      </c>
-      <c r="G10">
-        <v>40</v>
-      </c>
-      <c r="H10">
-        <v>31</v>
-      </c>
-      <c r="I10">
-        <v>44</v>
-      </c>
-      <c r="J10">
-        <v>43</v>
-      </c>
-      <c r="K10">
-        <v>57</v>
-      </c>
-      <c r="L10">
-        <v>40</v>
-      </c>
-      <c r="M10">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-17
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -9,20 +9,20 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Albany Park" sheetId="3" r:id="rId3"/>
-    <sheet name="Woodlawn" sheetId="4" r:id="rId4"/>
+    <sheet name="Austin" sheetId="3" r:id="rId3"/>
+    <sheet name="Roseland" sheetId="4" r:id="rId4"/>
     <sheet name="North Lawndale" sheetId="5" r:id="rId5"/>
-    <sheet name="Englewood" sheetId="6" r:id="rId6"/>
-    <sheet name="Roseland" sheetId="7" r:id="rId7"/>
-    <sheet name="South Shore" sheetId="8" r:id="rId8"/>
-    <sheet name="Old Town" sheetId="9" r:id="rId9"/>
-    <sheet name="Loop" sheetId="10" r:id="rId10"/>
-    <sheet name="Lincoln Park" sheetId="11" r:id="rId11"/>
-    <sheet name="O'Hare" sheetId="12" r:id="rId12"/>
-    <sheet name="Near South Side" sheetId="13" r:id="rId13"/>
-    <sheet name="Logan Square" sheetId="14" r:id="rId14"/>
-    <sheet name="Grand Crossing" sheetId="15" r:id="rId15"/>
-    <sheet name="Austin" sheetId="16" r:id="rId16"/>
+    <sheet name="Albany Park" sheetId="6" r:id="rId6"/>
+    <sheet name="Woodlawn" sheetId="7" r:id="rId7"/>
+    <sheet name="Englewood" sheetId="8" r:id="rId8"/>
+    <sheet name="South Shore" sheetId="9" r:id="rId9"/>
+    <sheet name="Old Town" sheetId="10" r:id="rId10"/>
+    <sheet name="Loop" sheetId="11" r:id="rId11"/>
+    <sheet name="Lincoln Park" sheetId="12" r:id="rId12"/>
+    <sheet name="O'Hare" sheetId="13" r:id="rId13"/>
+    <sheet name="Near South Side" sheetId="14" r:id="rId14"/>
+    <sheet name="Logan Square" sheetId="15" r:id="rId15"/>
+    <sheet name="Grand Crossing" sheetId="16" r:id="rId16"/>
     <sheet name="Avondale" sheetId="17" r:id="rId17"/>
     <sheet name="Rush &amp; Division" sheetId="18" r:id="rId18"/>
     <sheet name="Chatham" sheetId="19" r:id="rId19"/>
@@ -946,7 +946,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1039,7 +1039,7 @@
         <v>25</v>
       </c>
       <c r="M6">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>828</v>
+        <v>831</v>
       </c>
     </row>
   </sheetData>
@@ -1247,6 +1247,272 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>17</v>
+      </c>
+      <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>17</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>17</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>26</v>
+      </c>
+      <c r="D7">
+        <v>44</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>79</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>13</v>
+      </c>
+      <c r="I7">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>9</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>53</v>
+      </c>
+      <c r="E8">
+        <v>76</v>
+      </c>
+      <c r="F8">
+        <v>103</v>
+      </c>
+      <c r="G8">
+        <v>39</v>
+      </c>
+      <c r="H8">
+        <v>30</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>29</v>
+      </c>
+      <c r="K8">
+        <v>33</v>
+      </c>
+      <c r="L8">
+        <v>17</v>
+      </c>
+      <c r="M8">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1600,7 +1866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1833,257 +2099,6 @@
       </c>
       <c r="M7">
         <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>47</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>22</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2156,23 +2171,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2">
         <v>2</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -2182,42 +2200,42 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J4">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
@@ -2225,8 +2243,8 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K5">
-        <v>1</v>
+      <c r="L5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2234,40 +2252,22 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>4</v>
       </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
       <c r="H6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2275,40 +2275,40 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D7">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I7">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
         <v>12</v>
       </c>
-      <c r="L7">
-        <v>10</v>
-      </c>
       <c r="M7">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2316,40 +2316,40 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C8">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D8">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F8">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>22</v>
+      </c>
+      <c r="L8">
+        <v>21</v>
+      </c>
+      <c r="M8">
         <v>17</v>
-      </c>
-      <c r="H8">
-        <v>15</v>
-      </c>
-      <c r="I8">
-        <v>27</v>
-      </c>
-      <c r="J8">
-        <v>19</v>
-      </c>
-      <c r="K8">
-        <v>20</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="M8">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2422,35 +2422,35 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
+      <c r="F2">
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
       <c r="C3">
         <v>1</v>
       </c>
@@ -2458,21 +2458,24 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -2480,27 +2483,15 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
       <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="L4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5">
         <v>1</v>
       </c>
     </row>
@@ -2509,40 +2500,40 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
         <v>8</v>
       </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
       <c r="J6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2550,40 +2541,40 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C7">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D7">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="E7">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F7">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I7">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J7">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K7">
+        <v>12</v>
+      </c>
+      <c r="L7">
         <v>10</v>
       </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
       <c r="M7">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2591,40 +2582,40 @@
         <v>10</v>
       </c>
       <c r="B8">
+        <v>29</v>
+      </c>
+      <c r="C8">
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>26</v>
+      </c>
+      <c r="F8">
+        <v>28</v>
+      </c>
+      <c r="G8">
+        <v>17</v>
+      </c>
+      <c r="H8">
+        <v>15</v>
+      </c>
+      <c r="I8">
+        <v>27</v>
+      </c>
+      <c r="J8">
         <v>19</v>
-      </c>
-      <c r="C8">
-        <v>32</v>
-      </c>
-      <c r="D8">
-        <v>42</v>
-      </c>
-      <c r="E8">
-        <v>37</v>
-      </c>
-      <c r="F8">
-        <v>23</v>
-      </c>
-      <c r="G8">
-        <v>26</v>
-      </c>
-      <c r="H8">
-        <v>18</v>
-      </c>
-      <c r="I8">
-        <v>23</v>
-      </c>
-      <c r="J8">
-        <v>31</v>
       </c>
       <c r="K8">
         <v>20</v>
       </c>
       <c r="L8">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2634,7 +2625,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -2697,40 +2688,28 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>4</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
         <v>5</v>
       </c>
     </row>
@@ -2738,74 +2717,95 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K3">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>13</v>
-      </c>
-      <c r="M3">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="J5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>7</v>
+      </c>
+      <c r="L6">
+        <v>7</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -2813,145 +2813,84 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>31</v>
+      </c>
+      <c r="F7">
+        <v>18</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>32</v>
+      </c>
+      <c r="D8">
+        <v>42</v>
+      </c>
+      <c r="E8">
+        <v>37</v>
+      </c>
+      <c r="F8">
+        <v>23</v>
+      </c>
+      <c r="G8">
+        <v>26</v>
+      </c>
+      <c r="H8">
+        <v>18</v>
+      </c>
+      <c r="I8">
+        <v>23</v>
+      </c>
+      <c r="J8">
+        <v>31</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>26</v>
+      </c>
+      <c r="M8">
         <v>8</v>
-      </c>
-      <c r="B8">
-        <v>24</v>
-      </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>21</v>
-      </c>
-      <c r="E8">
-        <v>22</v>
-      </c>
-      <c r="F8">
-        <v>27</v>
-      </c>
-      <c r="G8">
-        <v>15</v>
-      </c>
-      <c r="H8">
-        <v>25</v>
-      </c>
-      <c r="I8">
-        <v>21</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>49</v>
-      </c>
-      <c r="L8">
-        <v>44</v>
-      </c>
-      <c r="M8">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>45</v>
-      </c>
-      <c r="C9">
-        <v>64</v>
-      </c>
-      <c r="D9">
-        <v>46</v>
-      </c>
-      <c r="E9">
-        <v>50</v>
-      </c>
-      <c r="F9">
-        <v>38</v>
-      </c>
-      <c r="G9">
-        <v>19</v>
-      </c>
-      <c r="H9">
-        <v>27</v>
-      </c>
-      <c r="I9">
-        <v>37</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>35</v>
-      </c>
-      <c r="L9">
-        <v>35</v>
-      </c>
-      <c r="M9">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>77</v>
-      </c>
-      <c r="C10">
-        <v>106</v>
-      </c>
-      <c r="D10">
-        <v>82</v>
-      </c>
-      <c r="E10">
-        <v>88</v>
-      </c>
-      <c r="F10">
-        <v>91</v>
-      </c>
-      <c r="G10">
-        <v>47</v>
-      </c>
-      <c r="H10">
-        <v>66</v>
-      </c>
-      <c r="I10">
-        <v>77</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>110</v>
-      </c>
-      <c r="L10">
-        <v>98</v>
-      </c>
-      <c r="M10">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -3025,31 +2964,31 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K2">
         <v>7</v>
@@ -3058,7 +2997,7 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3066,40 +3005,40 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H3">
         <v>8</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3109,43 +3048,52 @@
       <c r="I4">
         <v>1</v>
       </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="M6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
       </c>
       <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <v>1</v>
       </c>
     </row>
@@ -3154,40 +3102,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D8">
+        <v>21</v>
+      </c>
+      <c r="E8">
         <v>22</v>
       </c>
-      <c r="E8">
-        <v>44</v>
-      </c>
       <c r="F8">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I8">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="J8">
         <v>26</v>
       </c>
       <c r="K8">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="L8">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="M8">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3195,40 +3143,40 @@
         <v>9</v>
       </c>
       <c r="B9">
+        <v>45</v>
+      </c>
+      <c r="C9">
+        <v>64</v>
+      </c>
+      <c r="D9">
         <v>46</v>
       </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
       <c r="E9">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="F9">
-        <v>114</v>
+        <v>38</v>
       </c>
       <c r="G9">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="I9">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="J9">
         <v>20</v>
       </c>
       <c r="K9">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="L9">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3236,40 +3184,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D10">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E10">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="F10">
-        <v>167</v>
+        <v>91</v>
       </c>
       <c r="G10">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="H10">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="I10">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J10">
         <v>67</v>
       </c>
       <c r="K10">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="L10">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="M10">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -4423,7 +4371,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6556,7 +6504,7 @@
         <v>25</v>
       </c>
       <c r="M65">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -7027,7 +6975,7 @@
         <v>62</v>
       </c>
       <c r="M77">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -7890,7 +7838,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>828</v>
+        <v>831</v>
       </c>
     </row>
   </sheetData>
@@ -10454,7 +10402,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -10517,29 +10465,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -10547,68 +10507,68 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5">
         <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>2</v>
@@ -10616,84 +10576,141 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>31</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
+        <v>44</v>
+      </c>
+      <c r="F8">
+        <v>38</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8">
+        <v>50</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>24</v>
+      </c>
+      <c r="L8">
+        <v>14</v>
+      </c>
+      <c r="M8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>59</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="E9">
+        <v>73</v>
+      </c>
+      <c r="F9">
+        <v>114</v>
+      </c>
+      <c r="G9">
+        <v>58</v>
+      </c>
+      <c r="H9">
+        <v>41</v>
+      </c>
+      <c r="I9">
+        <v>44</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>25</v>
+      </c>
+      <c r="L9">
+        <v>27</v>
+      </c>
+      <c r="M9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>15</v>
-      </c>
-      <c r="D7">
-        <v>13</v>
-      </c>
-      <c r="E7">
-        <v>13</v>
-      </c>
-      <c r="F7">
-        <v>10</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>14</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
+      <c r="B10">
+        <v>78</v>
+      </c>
+      <c r="C10">
+        <v>99</v>
+      </c>
+      <c r="D10">
+        <v>65</v>
+      </c>
+      <c r="E10">
+        <v>130</v>
+      </c>
+      <c r="F10">
+        <v>167</v>
+      </c>
+      <c r="G10">
+        <v>92</v>
+      </c>
+      <c r="H10">
+        <v>104</v>
+      </c>
+      <c r="I10">
+        <v>89</v>
+      </c>
+      <c r="J10">
+        <v>67</v>
+      </c>
+      <c r="K10">
+        <v>71</v>
+      </c>
+      <c r="L10">
+        <v>61</v>
+      </c>
+      <c r="M10">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -13430,7 +13447,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13494,21 +13511,39 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
       </c>
       <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -13517,168 +13552,213 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
         <v>5</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D6">
-        <v>17</v>
-      </c>
-      <c r="E6">
-        <v>14</v>
-      </c>
-      <c r="F6">
-        <v>15</v>
-      </c>
-      <c r="G6">
-        <v>6</v>
-      </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
-      <c r="I6">
-        <v>6</v>
-      </c>
-      <c r="J6">
-        <v>8</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>14</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="H8">
+        <v>19</v>
+      </c>
+      <c r="I8">
+        <v>29</v>
+      </c>
+      <c r="J8">
+        <v>19</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>26</v>
+      </c>
+      <c r="M8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>56</v>
+      </c>
+      <c r="C9">
+        <v>45</v>
+      </c>
+      <c r="D9">
+        <v>42</v>
+      </c>
+      <c r="E9">
+        <v>51</v>
+      </c>
+      <c r="F9">
+        <v>54</v>
+      </c>
+      <c r="G9">
+        <v>32</v>
+      </c>
+      <c r="H9">
+        <v>29</v>
+      </c>
+      <c r="I9">
+        <v>35</v>
+      </c>
+      <c r="J9">
+        <v>40</v>
+      </c>
+      <c r="K9">
+        <v>37</v>
+      </c>
+      <c r="L9">
+        <v>25</v>
+      </c>
+      <c r="M9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>33</v>
-      </c>
-      <c r="C7">
-        <v>23</v>
-      </c>
-      <c r="D7">
+      <c r="B10">
+        <v>82</v>
+      </c>
+      <c r="C10">
+        <v>70</v>
+      </c>
+      <c r="D10">
+        <v>59</v>
+      </c>
+      <c r="E10">
+        <v>74</v>
+      </c>
+      <c r="F10">
+        <v>77</v>
+      </c>
+      <c r="G10">
+        <v>56</v>
+      </c>
+      <c r="H10">
+        <v>60</v>
+      </c>
+      <c r="I10">
+        <v>82</v>
+      </c>
+      <c r="J10">
+        <v>76</v>
+      </c>
+      <c r="K10">
+        <v>68</v>
+      </c>
+      <c r="L10">
+        <v>62</v>
+      </c>
+      <c r="M10">
         <v>27</v>
-      </c>
-      <c r="E7">
-        <v>25</v>
-      </c>
-      <c r="F7">
-        <v>22</v>
-      </c>
-      <c r="G7">
-        <v>13</v>
-      </c>
-      <c r="H7">
-        <v>11</v>
-      </c>
-      <c r="I7">
-        <v>17</v>
-      </c>
-      <c r="J7">
-        <v>19</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
-      <c r="M7">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -16286,7 +16366,7 @@
         <v>7</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -16327,7 +16407,7 @@
         <v>25</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -18706,7 +18786,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -18769,38 +18849,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
-        <v>6</v>
-      </c>
-      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>7</v>
-      </c>
-      <c r="H2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -18808,53 +18879,32 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
-      </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>11</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+      <c r="E4">
         <v>2</v>
       </c>
       <c r="J4">
@@ -18862,157 +18912,120 @@
       </c>
       <c r="K4">
         <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
         <v>1</v>
       </c>
       <c r="I5">
         <v>1</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>13</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>12</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>34</v>
-      </c>
-      <c r="C7">
-        <v>45</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>42</v>
-      </c>
-      <c r="G7">
-        <v>32</v>
-      </c>
-      <c r="H7">
-        <v>26</v>
-      </c>
-      <c r="I7">
-        <v>21</v>
-      </c>
       <c r="J7">
+        <v>14</v>
+      </c>
+      <c r="K7">
         <v>15</v>
       </c>
-      <c r="K7">
-        <v>44</v>
-      </c>
       <c r="L7">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>71</v>
-      </c>
-      <c r="C8">
-        <v>91</v>
-      </c>
-      <c r="D8">
-        <v>57</v>
-      </c>
-      <c r="E8">
-        <v>65</v>
-      </c>
-      <c r="F8">
-        <v>75</v>
-      </c>
-      <c r="G8">
-        <v>41</v>
-      </c>
-      <c r="H8">
-        <v>29</v>
-      </c>
-      <c r="I8">
-        <v>45</v>
-      </c>
-      <c r="J8">
-        <v>31</v>
-      </c>
-      <c r="K8">
-        <v>27</v>
-      </c>
-      <c r="L8">
-        <v>32</v>
-      </c>
-      <c r="M8">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>111</v>
-      </c>
-      <c r="C9">
-        <v>142</v>
-      </c>
-      <c r="D9">
-        <v>107</v>
-      </c>
-      <c r="E9">
-        <v>98</v>
-      </c>
-      <c r="F9">
-        <v>138</v>
-      </c>
-      <c r="G9">
-        <v>92</v>
-      </c>
-      <c r="H9">
-        <v>76</v>
-      </c>
-      <c r="I9">
-        <v>90</v>
-      </c>
-      <c r="J9">
-        <v>69</v>
-      </c>
-      <c r="K9">
-        <v>95</v>
-      </c>
-      <c r="L9">
-        <v>103</v>
-      </c>
-      <c r="M9">
-        <v>35</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -21055,7 +21068,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -21119,39 +21132,21 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>7</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -21160,213 +21155,168 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
         <v>5</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J3">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>7</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
         <v>6</v>
       </c>
-      <c r="D6">
-        <v>1</v>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>33</v>
+      </c>
+      <c r="C7">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>27</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
+      </c>
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7">
+        <v>17</v>
       </c>
       <c r="J7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
         <v>19</v>
       </c>
-      <c r="C8">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>11</v>
-      </c>
-      <c r="E8">
-        <v>14</v>
-      </c>
-      <c r="F8">
-        <v>12</v>
-      </c>
-      <c r="G8">
-        <v>14</v>
-      </c>
-      <c r="H8">
-        <v>19</v>
-      </c>
-      <c r="I8">
-        <v>29</v>
-      </c>
-      <c r="J8">
-        <v>19</v>
-      </c>
-      <c r="K8">
-        <v>20</v>
-      </c>
-      <c r="L8">
-        <v>26</v>
-      </c>
-      <c r="M8">
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>56</v>
-      </c>
-      <c r="C9">
-        <v>45</v>
-      </c>
-      <c r="D9">
-        <v>42</v>
-      </c>
-      <c r="E9">
-        <v>51</v>
-      </c>
-      <c r="F9">
-        <v>54</v>
-      </c>
-      <c r="G9">
-        <v>32</v>
-      </c>
-      <c r="H9">
-        <v>29</v>
-      </c>
-      <c r="I9">
-        <v>35</v>
-      </c>
-      <c r="J9">
-        <v>40</v>
-      </c>
-      <c r="K9">
-        <v>37</v>
-      </c>
-      <c r="L9">
-        <v>25</v>
-      </c>
-      <c r="M9">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
+      <c r="M7">
         <v>10</v>
-      </c>
-      <c r="B10">
-        <v>82</v>
-      </c>
-      <c r="C10">
-        <v>70</v>
-      </c>
-      <c r="D10">
-        <v>59</v>
-      </c>
-      <c r="E10">
-        <v>74</v>
-      </c>
-      <c r="F10">
-        <v>77</v>
-      </c>
-      <c r="G10">
-        <v>56</v>
-      </c>
-      <c r="H10">
-        <v>60</v>
-      </c>
-      <c r="I10">
-        <v>82</v>
-      </c>
-      <c r="J10">
-        <v>76</v>
-      </c>
-      <c r="K10">
-        <v>68</v>
-      </c>
-      <c r="L10">
-        <v>62</v>
-      </c>
-      <c r="M10">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -23214,10 +23164,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -23277,41 +23227,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -23319,75 +23266,60 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B4">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>6</v>
-      </c>
-      <c r="E4">
-        <v>7</v>
-      </c>
-      <c r="F4">
-        <v>7</v>
-      </c>
-      <c r="G4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -23398,84 +23330,147 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <v>16</v>
-      </c>
-      <c r="D5">
-        <v>22</v>
-      </c>
-      <c r="E5">
-        <v>14</v>
-      </c>
-      <c r="F5">
-        <v>13</v>
-      </c>
-      <c r="G5">
         <v>6</v>
       </c>
       <c r="H5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>13</v>
-      </c>
-      <c r="K5">
-        <v>8</v>
-      </c>
-      <c r="L5">
-        <v>7</v>
-      </c>
-      <c r="M5">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>45</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>42</v>
+      </c>
+      <c r="G7">
+        <v>32</v>
+      </c>
+      <c r="H7">
+        <v>26</v>
+      </c>
+      <c r="I7">
+        <v>21</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>44</v>
+      </c>
+      <c r="L7">
+        <v>44</v>
+      </c>
+      <c r="M7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>71</v>
+      </c>
+      <c r="C8">
+        <v>91</v>
+      </c>
+      <c r="D8">
+        <v>57</v>
+      </c>
+      <c r="E8">
+        <v>65</v>
+      </c>
+      <c r="F8">
+        <v>75</v>
+      </c>
+      <c r="G8">
+        <v>41</v>
+      </c>
+      <c r="H8">
+        <v>29</v>
+      </c>
+      <c r="I8">
+        <v>45</v>
+      </c>
+      <c r="J8">
+        <v>31</v>
+      </c>
+      <c r="K8">
+        <v>27</v>
+      </c>
+      <c r="L8">
+        <v>32</v>
+      </c>
+      <c r="M8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>30</v>
-      </c>
-      <c r="C6">
-        <v>31</v>
-      </c>
-      <c r="D6">
-        <v>34</v>
-      </c>
-      <c r="E6">
-        <v>25</v>
-      </c>
-      <c r="F6">
-        <v>25</v>
-      </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>22</v>
-      </c>
-      <c r="I6">
-        <v>16</v>
-      </c>
-      <c r="J6">
-        <v>28</v>
-      </c>
-      <c r="K6">
-        <v>17</v>
-      </c>
-      <c r="L6">
-        <v>16</v>
-      </c>
-      <c r="M6">
-        <v>13</v>
+      <c r="B9">
+        <v>111</v>
+      </c>
+      <c r="C9">
+        <v>142</v>
+      </c>
+      <c r="D9">
+        <v>107</v>
+      </c>
+      <c r="E9">
+        <v>98</v>
+      </c>
+      <c r="F9">
+        <v>138</v>
+      </c>
+      <c r="G9">
+        <v>92</v>
+      </c>
+      <c r="H9">
+        <v>76</v>
+      </c>
+      <c r="I9">
+        <v>90</v>
+      </c>
+      <c r="J9">
+        <v>69</v>
+      </c>
+      <c r="K9">
+        <v>95</v>
+      </c>
+      <c r="L9">
+        <v>103</v>
+      </c>
+      <c r="M9">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -25266,10 +25261,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -25329,26 +25324,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L2">
         <v>2</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -25356,173 +25366,163 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I3">
         <v>2</v>
       </c>
       <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3">
         <v>6</v>
       </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-      <c r="L3">
+      <c r="M3">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>7</v>
+      </c>
+      <c r="G4">
+        <v>7</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+      <c r="J4">
+        <v>12</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>22</v>
+      </c>
+      <c r="E5">
+        <v>14</v>
+      </c>
+      <c r="F5">
+        <v>13</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>11</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="K5">
+        <v>8</v>
+      </c>
+      <c r="L5">
+        <v>7</v>
+      </c>
+      <c r="M5">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E6">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F6">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="K6">
         <v>17</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="M6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>26</v>
-      </c>
-      <c r="D7">
-        <v>44</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>79</v>
-      </c>
-      <c r="G7">
-        <v>24</v>
-      </c>
-      <c r="H7">
         <v>13</v>
-      </c>
-      <c r="I7">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>9</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>27</v>
-      </c>
-      <c r="C8">
-        <v>37</v>
-      </c>
-      <c r="D8">
-        <v>53</v>
-      </c>
-      <c r="E8">
-        <v>76</v>
-      </c>
-      <c r="F8">
-        <v>103</v>
-      </c>
-      <c r="G8">
-        <v>39</v>
-      </c>
-      <c r="H8">
-        <v>30</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>29</v>
-      </c>
-      <c r="K8">
-        <v>33</v>
-      </c>
-      <c r="L8">
-        <v>17</v>
-      </c>
-      <c r="M8">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-26
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -9,28 +9,28 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="River North" sheetId="3" r:id="rId3"/>
-    <sheet name="North Lawndale" sheetId="4" r:id="rId4"/>
-    <sheet name="Englewood" sheetId="5" r:id="rId5"/>
-    <sheet name="Uptown" sheetId="6" r:id="rId6"/>
-    <sheet name="Loop" sheetId="7" r:id="rId7"/>
-    <sheet name="Logan Square" sheetId="8" r:id="rId8"/>
-    <sheet name="Riverdale" sheetId="9" r:id="rId9"/>
-    <sheet name="Fuller Park" sheetId="10" r:id="rId10"/>
-    <sheet name="Little Village" sheetId="11" r:id="rId11"/>
-    <sheet name="Chatham" sheetId="12" r:id="rId12"/>
-    <sheet name="West Loop" sheetId="13" r:id="rId13"/>
-    <sheet name="Auburn Gresham" sheetId="14" r:id="rId14"/>
-    <sheet name="Lake View" sheetId="15" r:id="rId15"/>
-    <sheet name="Humboldt Park" sheetId="16" r:id="rId16"/>
-    <sheet name="Austin" sheetId="17" r:id="rId17"/>
-    <sheet name="Roseland" sheetId="18" r:id="rId18"/>
-    <sheet name="Albany Park" sheetId="19" r:id="rId19"/>
-    <sheet name="Woodlawn" sheetId="20" r:id="rId20"/>
-    <sheet name="South Shore" sheetId="21" r:id="rId21"/>
-    <sheet name="Old Town" sheetId="22" r:id="rId22"/>
-    <sheet name="Lincoln Park" sheetId="23" r:id="rId23"/>
-    <sheet name="O'Hare" sheetId="24" r:id="rId24"/>
+    <sheet name="O'Hare" sheetId="3" r:id="rId3"/>
+    <sheet name="River North" sheetId="4" r:id="rId4"/>
+    <sheet name="North Lawndale" sheetId="5" r:id="rId5"/>
+    <sheet name="Englewood" sheetId="6" r:id="rId6"/>
+    <sheet name="Uptown" sheetId="7" r:id="rId7"/>
+    <sheet name="Loop" sheetId="8" r:id="rId8"/>
+    <sheet name="Logan Square" sheetId="9" r:id="rId9"/>
+    <sheet name="Riverdale" sheetId="10" r:id="rId10"/>
+    <sheet name="Fuller Park" sheetId="11" r:id="rId11"/>
+    <sheet name="Little Village" sheetId="12" r:id="rId12"/>
+    <sheet name="Chatham" sheetId="13" r:id="rId13"/>
+    <sheet name="West Loop" sheetId="14" r:id="rId14"/>
+    <sheet name="Auburn Gresham" sheetId="15" r:id="rId15"/>
+    <sheet name="Lake View" sheetId="16" r:id="rId16"/>
+    <sheet name="Humboldt Park" sheetId="17" r:id="rId17"/>
+    <sheet name="Austin" sheetId="18" r:id="rId18"/>
+    <sheet name="Roseland" sheetId="19" r:id="rId19"/>
+    <sheet name="Albany Park" sheetId="20" r:id="rId20"/>
+    <sheet name="Woodlawn" sheetId="21" r:id="rId21"/>
+    <sheet name="South Shore" sheetId="22" r:id="rId22"/>
+    <sheet name="Old Town" sheetId="23" r:id="rId23"/>
+    <sheet name="Lincoln Park" sheetId="24" r:id="rId24"/>
     <sheet name="Near South Side" sheetId="25" r:id="rId25"/>
     <sheet name="Grand Crossing" sheetId="26" r:id="rId26"/>
     <sheet name="Avondale" sheetId="27" r:id="rId27"/>
@@ -1039,7 +1039,7 @@
         <v>25</v>
       </c>
       <c r="M6">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1247,6 +1247,183 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1526,7 +1703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1769,7 +1946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2084,7 +2261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2370,7 +2547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2643,7 +2820,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2939,7 +3116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3224,324 +3401,6 @@
       </c>
       <c r="M9">
         <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>8</v>
-      </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <v>7</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-      <c r="K3">
-        <v>12</v>
-      </c>
-      <c r="L3">
-        <v>14</v>
-      </c>
-      <c r="M3">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>23</v>
-      </c>
-      <c r="C8">
-        <v>31</v>
-      </c>
-      <c r="D8">
-        <v>22</v>
-      </c>
-      <c r="E8">
-        <v>44</v>
-      </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>24</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="M8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>46</v>
-      </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>73</v>
-      </c>
-      <c r="F9">
-        <v>114</v>
-      </c>
-      <c r="G9">
-        <v>58</v>
-      </c>
-      <c r="H9">
-        <v>41</v>
-      </c>
-      <c r="I9">
-        <v>44</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>25</v>
-      </c>
-      <c r="L9">
-        <v>27</v>
-      </c>
-      <c r="M9">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>78</v>
-      </c>
-      <c r="C10">
-        <v>99</v>
-      </c>
-      <c r="D10">
-        <v>65</v>
-      </c>
-      <c r="E10">
-        <v>130</v>
-      </c>
-      <c r="F10">
-        <v>167</v>
-      </c>
-      <c r="G10">
-        <v>92</v>
-      </c>
-      <c r="H10">
-        <v>104</v>
-      </c>
-      <c r="I10">
-        <v>89</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>71</v>
-      </c>
-      <c r="L10">
-        <v>61</v>
-      </c>
-      <c r="M10">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -3615,40 +3474,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2">
         <v>7</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
       <c r="L2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3656,47 +3515,47 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
         <v>7</v>
       </c>
-      <c r="G3">
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
         <v>6</v>
       </c>
-      <c r="H3">
-        <v>6</v>
-      </c>
-      <c r="I3">
-        <v>9</v>
-      </c>
       <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>14</v>
       </c>
-      <c r="K3">
-        <v>7</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
       <c r="M3">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
@@ -3704,33 +3563,30 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D6">
+      <c r="K6">
         <v>1</v>
       </c>
     </row>
@@ -3738,7 +3594,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>1</v>
       </c>
     </row>
@@ -3747,40 +3603,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C8">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D8">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E8">
+        <v>44</v>
+      </c>
+      <c r="F8">
+        <v>38</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8">
+        <v>50</v>
+      </c>
+      <c r="I8">
+        <v>34</v>
+      </c>
+      <c r="J8">
+        <v>26</v>
+      </c>
+      <c r="K8">
+        <v>24</v>
+      </c>
+      <c r="L8">
         <v>14</v>
       </c>
-      <c r="F8">
-        <v>12</v>
-      </c>
-      <c r="G8">
-        <v>14</v>
-      </c>
-      <c r="H8">
-        <v>19</v>
-      </c>
-      <c r="I8">
-        <v>29</v>
-      </c>
-      <c r="J8">
-        <v>19</v>
-      </c>
-      <c r="K8">
-        <v>20</v>
-      </c>
-      <c r="L8">
-        <v>26</v>
-      </c>
       <c r="M8">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3788,40 +3644,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D9">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E9">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="F9">
-        <v>54</v>
+        <v>114</v>
       </c>
       <c r="G9">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="H9">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="I9">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K9">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3829,40 +3685,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C10">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E10">
-        <v>74</v>
+        <v>130</v>
       </c>
       <c r="F10">
-        <v>77</v>
+        <v>167</v>
       </c>
       <c r="G10">
-        <v>56</v>
+        <v>92</v>
       </c>
       <c r="H10">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="I10">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="J10">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="K10">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L10">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M10">
-        <v>27</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -3872,7 +3728,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -3935,29 +3791,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3965,153 +3833,213 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="H3">
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="K3">
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>9</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
-      <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>14</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="H8">
+        <v>19</v>
+      </c>
+      <c r="I8">
+        <v>29</v>
+      </c>
+      <c r="J8">
+        <v>19</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>26</v>
+      </c>
+      <c r="M8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>56</v>
+      </c>
+      <c r="C9">
+        <v>45</v>
+      </c>
+      <c r="D9">
+        <v>42</v>
+      </c>
+      <c r="E9">
+        <v>51</v>
+      </c>
+      <c r="F9">
+        <v>54</v>
+      </c>
+      <c r="G9">
+        <v>32</v>
+      </c>
+      <c r="H9">
+        <v>29</v>
+      </c>
+      <c r="I9">
+        <v>35</v>
+      </c>
+      <c r="J9">
+        <v>40</v>
+      </c>
+      <c r="K9">
+        <v>37</v>
+      </c>
+      <c r="L9">
+        <v>25</v>
+      </c>
+      <c r="M9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>15</v>
-      </c>
-      <c r="D7">
-        <v>13</v>
-      </c>
-      <c r="E7">
-        <v>13</v>
-      </c>
-      <c r="F7">
-        <v>10</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>14</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>6</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
+      <c r="B10">
+        <v>82</v>
+      </c>
+      <c r="C10">
+        <v>70</v>
+      </c>
+      <c r="D10">
+        <v>59</v>
+      </c>
+      <c r="E10">
+        <v>74</v>
+      </c>
+      <c r="F10">
+        <v>77</v>
+      </c>
+      <c r="G10">
+        <v>56</v>
+      </c>
+      <c r="H10">
+        <v>60</v>
+      </c>
+      <c r="I10">
+        <v>82</v>
+      </c>
+      <c r="J10">
+        <v>76</v>
+      </c>
+      <c r="K10">
+        <v>68</v>
+      </c>
+      <c r="L10">
+        <v>62</v>
+      </c>
+      <c r="M10">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -4560,7 +4488,7 @@
         <v>3</v>
       </c>
       <c r="M11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6135,7 +6063,7 @@
         <v>196</v>
       </c>
       <c r="M53">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -6412,7 +6340,7 @@
         <v>16</v>
       </c>
       <c r="M61">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -6699,7 +6627,7 @@
         <v>21</v>
       </c>
       <c r="M68">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -7050,7 +6978,7 @@
         <v>62</v>
       </c>
       <c r="M77">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -8086,23 +8014,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
       <c r="L2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -8110,44 +8044,38 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
       <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>5</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
@@ -8156,36 +8084,27 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>7</v>
-      </c>
-      <c r="L5">
         <v>4</v>
       </c>
       <c r="M5">
@@ -8197,40 +8116,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C6">
+        <v>13</v>
+      </c>
+      <c r="D6">
         <v>10</v>
       </c>
-      <c r="D6">
-        <v>17</v>
-      </c>
       <c r="E6">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
         <v>8</v>
       </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
       <c r="L6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -8238,31 +8157,31 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F7">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K7">
         <v>15</v>
@@ -8271,7 +8190,7 @@
         <v>6</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8280,6 +8199,264 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>6</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>33</v>
+      </c>
+      <c r="C7">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>27</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
+      </c>
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7">
+        <v>17</v>
+      </c>
+      <c r="J7">
+        <v>19</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7">
+        <v>6</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8550,7 +8727,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8816,7 +8993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9049,257 +9226,6 @@
       </c>
       <c r="M7">
         <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>30</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
-      </c>
-      <c r="K7">
-        <v>17</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>47</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>12</v>
-      </c>
-      <c r="J8">
-        <v>18</v>
-      </c>
-      <c r="K8">
-        <v>22</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -10570,7 +10496,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -10633,32 +10559,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="B2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="H2">
         <v>2</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -10666,168 +10589,155 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5">
-        <v>7</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>13</v>
-      </c>
-      <c r="H5">
-        <v>11</v>
-      </c>
-      <c r="I5">
-        <v>14</v>
-      </c>
-      <c r="J5">
-        <v>12</v>
-      </c>
-      <c r="K5">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>6</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
-        <v>47</v>
-      </c>
-      <c r="C6">
-        <v>37</v>
-      </c>
-      <c r="D6">
-        <v>85</v>
-      </c>
-      <c r="E6">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>80</v>
-      </c>
-      <c r="G6">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>26</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="K6">
-        <v>19</v>
-      </c>
-      <c r="L6">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>50</v>
-      </c>
       <c r="C7">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="D7">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>82</v>
+        <v>30</v>
       </c>
       <c r="F7">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="G7">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
+        <v>17</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
+      </c>
+      <c r="M7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8">
+        <v>47</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>12</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>22</v>
+      </c>
+      <c r="L8">
         <v>21</v>
       </c>
-      <c r="I7">
-        <v>47</v>
-      </c>
-      <c r="J7">
-        <v>33</v>
-      </c>
-      <c r="K7">
-        <v>34</v>
-      </c>
-      <c r="L7">
-        <v>25</v>
-      </c>
-      <c r="M7">
-        <v>20</v>
+      <c r="M8">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -11231,7 +11141,7 @@
         <v>2</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -11272,7 +11182,7 @@
         <v>3</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -13139,7 +13049,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13202,11 +13112,8 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -13215,63 +13122,54 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
       </c>
       <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3">
         <v>5</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M3">
         <v>3</v>
@@ -13279,147 +13177,136 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="J4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>13</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="I5">
+        <v>14</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="K5">
+        <v>9</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6">
+        <v>47</v>
+      </c>
+      <c r="C6">
+        <v>37</v>
+      </c>
+      <c r="D6">
+        <v>85</v>
+      </c>
+      <c r="E6">
+        <v>75</v>
+      </c>
+      <c r="F6">
+        <v>80</v>
+      </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>26</v>
+      </c>
+      <c r="J6">
         <v>12</v>
       </c>
-      <c r="C6">
-        <v>21</v>
-      </c>
-      <c r="D6">
-        <v>28</v>
-      </c>
-      <c r="E6">
-        <v>21</v>
-      </c>
-      <c r="F6">
-        <v>35</v>
-      </c>
-      <c r="G6">
+      <c r="K6">
+        <v>19</v>
+      </c>
+      <c r="L6">
+        <v>11</v>
+      </c>
+      <c r="M6">
         <v>12</v>
-      </c>
-      <c r="H6">
-        <v>10</v>
-      </c>
-      <c r="I6">
-        <v>15</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>7</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="C7">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D7">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="E7">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="F7">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="G7">
+        <v>37</v>
+      </c>
+      <c r="H7">
+        <v>21</v>
+      </c>
+      <c r="I7">
+        <v>47</v>
+      </c>
+      <c r="J7">
+        <v>33</v>
+      </c>
+      <c r="K7">
+        <v>34</v>
+      </c>
+      <c r="L7">
         <v>25</v>
       </c>
-      <c r="H7">
-        <v>8</v>
-      </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>11</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
       <c r="M7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>32</v>
-      </c>
-      <c r="C8">
-        <v>61</v>
-      </c>
-      <c r="D8">
-        <v>78</v>
-      </c>
-      <c r="E8">
-        <v>68</v>
-      </c>
-      <c r="F8">
-        <v>100</v>
-      </c>
-      <c r="G8">
-        <v>43</v>
-      </c>
-      <c r="H8">
-        <v>26</v>
-      </c>
-      <c r="I8">
-        <v>32</v>
-      </c>
-      <c r="J8">
         <v>20</v>
-      </c>
-      <c r="K8">
-        <v>29</v>
-      </c>
-      <c r="L8">
-        <v>25</v>
-      </c>
-      <c r="M8">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -15981,7 +15868,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -16044,38 +15931,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>3</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -16083,211 +15973,182 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G3">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+      <c r="L3">
         <v>7</v>
       </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
-      </c>
-      <c r="L3">
-        <v>20</v>
-      </c>
       <c r="M3">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
+      <c r="I4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>21</v>
+      </c>
+      <c r="D6">
+        <v>28</v>
+      </c>
+      <c r="E6">
+        <v>21</v>
+      </c>
+      <c r="F6">
+        <v>35</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>15</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
         <v>7</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
+      <c r="M6">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>35</v>
+      </c>
+      <c r="D7">
+        <v>49</v>
+      </c>
+      <c r="E7">
+        <v>44</v>
+      </c>
+      <c r="F7">
+        <v>58</v>
+      </c>
+      <c r="G7">
+        <v>25</v>
+      </c>
+      <c r="H7">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>34</v>
-      </c>
-      <c r="C7">
-        <v>45</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>42</v>
-      </c>
-      <c r="G7">
-        <v>32</v>
-      </c>
-      <c r="H7">
-        <v>26</v>
-      </c>
       <c r="I7">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="C8">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="D8">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="E8">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F8">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G8">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H8">
+        <v>26</v>
+      </c>
+      <c r="I8">
+        <v>32</v>
+      </c>
+      <c r="J8">
+        <v>20</v>
+      </c>
+      <c r="K8">
         <v>29</v>
       </c>
-      <c r="I8">
-        <v>45</v>
-      </c>
-      <c r="J8">
-        <v>31</v>
-      </c>
-      <c r="K8">
-        <v>27</v>
-      </c>
       <c r="L8">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="M8">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>111</v>
-      </c>
-      <c r="C9">
-        <v>142</v>
-      </c>
-      <c r="D9">
-        <v>107</v>
-      </c>
-      <c r="E9">
-        <v>98</v>
-      </c>
-      <c r="F9">
-        <v>138</v>
-      </c>
-      <c r="G9">
-        <v>92</v>
-      </c>
-      <c r="H9">
-        <v>76</v>
-      </c>
-      <c r="I9">
-        <v>90</v>
-      </c>
-      <c r="J9">
-        <v>69</v>
-      </c>
-      <c r="K9">
-        <v>95</v>
-      </c>
-      <c r="L9">
-        <v>102</v>
-      </c>
-      <c r="M9">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -18577,76 +18438,76 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="L3">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="M3">
         <v>5</v>
@@ -18654,17 +18515,38 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -18672,7 +18554,10 @@
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="J6">
         <v>1</v>
       </c>
     </row>
@@ -18681,40 +18566,40 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="G7">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="L7">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -18722,40 +18607,40 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="C8">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="E8">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="F8">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="G8">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H8">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="J8">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="K8">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="L8">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -18763,40 +18648,40 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="C9">
-        <v>41</v>
+        <v>142</v>
       </c>
       <c r="D9">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="E9">
+        <v>98</v>
+      </c>
+      <c r="F9">
+        <v>138</v>
+      </c>
+      <c r="G9">
+        <v>92</v>
+      </c>
+      <c r="H9">
+        <v>76</v>
+      </c>
+      <c r="I9">
+        <v>90</v>
+      </c>
+      <c r="J9">
+        <v>69</v>
+      </c>
+      <c r="K9">
+        <v>95</v>
+      </c>
+      <c r="L9">
+        <v>102</v>
+      </c>
+      <c r="M9">
         <v>36</v>
-      </c>
-      <c r="F9">
-        <v>28</v>
-      </c>
-      <c r="G9">
-        <v>38</v>
-      </c>
-      <c r="H9">
-        <v>28</v>
-      </c>
-      <c r="I9">
-        <v>23</v>
-      </c>
-      <c r="J9">
-        <v>31</v>
-      </c>
-      <c r="K9">
-        <v>35</v>
-      </c>
-      <c r="L9">
-        <v>33</v>
-      </c>
-      <c r="M9">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -21120,7 +21005,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -21184,100 +21069,85 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>13</v>
-      </c>
       <c r="C3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="K3">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -21285,186 +21155,139 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+      <c r="B5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
+        <v>7</v>
+      </c>
+      <c r="C6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>9</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>14</v>
+      </c>
+      <c r="H7">
         <v>7</v>
       </c>
+      <c r="I7">
+        <v>4</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
       <c r="K7">
+        <v>11</v>
+      </c>
+      <c r="L7">
+        <v>8</v>
+      </c>
+      <c r="M7">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>30</v>
       </c>
       <c r="C8">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D8">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="E8">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="F8">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="G8">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="H8">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="I8">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="K8">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="L8">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="M8">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9">
-        <v>233</v>
+        <v>38</v>
       </c>
       <c r="C9">
-        <v>354</v>
+        <v>41</v>
       </c>
       <c r="D9">
-        <v>538</v>
+        <v>19</v>
       </c>
       <c r="E9">
-        <v>705</v>
+        <v>36</v>
       </c>
       <c r="F9">
-        <v>568</v>
+        <v>28</v>
       </c>
       <c r="G9">
-        <v>168</v>
+        <v>38</v>
       </c>
       <c r="H9">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="I9">
-        <v>194</v>
+        <v>23</v>
       </c>
       <c r="J9">
-        <v>122</v>
+        <v>31</v>
       </c>
       <c r="K9">
-        <v>114</v>
+        <v>35</v>
       </c>
       <c r="L9">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="M9">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>282</v>
-      </c>
-      <c r="C10">
-        <v>416</v>
-      </c>
-      <c r="D10">
-        <v>617</v>
-      </c>
-      <c r="E10">
-        <v>797</v>
-      </c>
-      <c r="F10">
-        <v>660</v>
-      </c>
-      <c r="G10">
-        <v>257</v>
-      </c>
-      <c r="H10">
-        <v>236</v>
-      </c>
-      <c r="I10">
-        <v>324</v>
-      </c>
-      <c r="J10">
-        <v>255</v>
-      </c>
-      <c r="K10">
-        <v>207</v>
-      </c>
-      <c r="L10">
-        <v>196</v>
-      </c>
-      <c r="M10">
-        <v>94</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -23208,7 +23031,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -23271,124 +23094,154 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
       </c>
       <c r="G2">
         <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>15</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>13</v>
+      </c>
       <c r="C3">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>34</v>
+      </c>
+      <c r="M3">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="G4">
         <v>1</v>
       </c>
       <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>8</v>
-      </c>
-      <c r="K6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -23396,84 +23249,133 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
-        <v>17</v>
-      </c>
-      <c r="C7">
-        <v>24</v>
-      </c>
-      <c r="D7">
-        <v>35</v>
-      </c>
-      <c r="E7">
-        <v>31</v>
-      </c>
-      <c r="F7">
-        <v>18</v>
-      </c>
-      <c r="G7">
-        <v>17</v>
-      </c>
-      <c r="H7">
-        <v>8</v>
-      </c>
-      <c r="I7">
-        <v>16</v>
-      </c>
-      <c r="J7">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K7">
-        <v>10</v>
-      </c>
-      <c r="L7">
-        <v>12</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>44</v>
+      </c>
+      <c r="D8">
+        <v>49</v>
+      </c>
+      <c r="E8">
+        <v>67</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8">
+        <v>57</v>
+      </c>
+      <c r="H8">
+        <v>80</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>64</v>
+      </c>
+      <c r="K8">
+        <v>48</v>
+      </c>
+      <c r="L8">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>233</v>
+      </c>
+      <c r="C9">
+        <v>354</v>
+      </c>
+      <c r="D9">
+        <v>538</v>
+      </c>
+      <c r="E9">
+        <v>705</v>
+      </c>
+      <c r="F9">
+        <v>568</v>
+      </c>
+      <c r="G9">
+        <v>168</v>
+      </c>
+      <c r="H9">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>194</v>
+      </c>
+      <c r="J9">
+        <v>122</v>
+      </c>
+      <c r="K9">
+        <v>114</v>
+      </c>
+      <c r="L9">
+        <v>95</v>
+      </c>
+      <c r="M9">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8">
-        <v>19</v>
-      </c>
-      <c r="C8">
-        <v>32</v>
-      </c>
-      <c r="D8">
-        <v>42</v>
-      </c>
-      <c r="E8">
-        <v>37</v>
-      </c>
-      <c r="F8">
-        <v>23</v>
-      </c>
-      <c r="G8">
-        <v>26</v>
-      </c>
-      <c r="H8">
-        <v>18</v>
-      </c>
-      <c r="I8">
-        <v>23</v>
-      </c>
-      <c r="J8">
-        <v>31</v>
-      </c>
-      <c r="K8">
-        <v>20</v>
-      </c>
-      <c r="L8">
-        <v>26</v>
-      </c>
-      <c r="M8">
-        <v>9</v>
+      <c r="B10">
+        <v>282</v>
+      </c>
+      <c r="C10">
+        <v>416</v>
+      </c>
+      <c r="D10">
+        <v>617</v>
+      </c>
+      <c r="E10">
+        <v>797</v>
+      </c>
+      <c r="F10">
+        <v>660</v>
+      </c>
+      <c r="G10">
+        <v>257</v>
+      </c>
+      <c r="H10">
+        <v>236</v>
+      </c>
+      <c r="I10">
+        <v>324</v>
+      </c>
+      <c r="J10">
+        <v>255</v>
+      </c>
+      <c r="K10">
+        <v>207</v>
+      </c>
+      <c r="L10">
+        <v>196</v>
+      </c>
+      <c r="M10">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -25367,10 +25269,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -25382,9 +25284,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -25407,33 +25310,54 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:12">
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -25441,100 +25365,176 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
       <c r="H3">
         <v>1</v>
       </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
       <c r="L3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>4</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="1" t="s">
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>7</v>
+      </c>
+      <c r="L6">
+        <v>7</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="1" t="s">
+      <c r="B7">
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <v>31</v>
+      </c>
+      <c r="F7">
+        <v>18</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>16</v>
+      </c>
+      <c r="J7">
+        <v>15</v>
+      </c>
+      <c r="K7">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>3</v>
-      </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>7</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>2</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
+      <c r="L7">
+        <v>12</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>32</v>
+      </c>
+      <c r="D8">
+        <v>42</v>
+      </c>
+      <c r="E8">
+        <v>37</v>
+      </c>
+      <c r="F8">
+        <v>23</v>
+      </c>
+      <c r="G8">
+        <v>26</v>
+      </c>
+      <c r="H8">
+        <v>18</v>
+      </c>
+      <c r="I8">
+        <v>23</v>
+      </c>
+      <c r="J8">
+        <v>31</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>26</v>
+      </c>
+      <c r="M8">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-05
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -47,18 +47,18 @@
     <sheet name="Sheffield &amp; DePaul" sheetId="38" r:id="rId38"/>
     <sheet name="Greektown" sheetId="39" r:id="rId39"/>
     <sheet name="River North" sheetId="40" r:id="rId40"/>
-    <sheet name="Roseland" sheetId="41" r:id="rId41"/>
-    <sheet name="Chinatown" sheetId="42" r:id="rId42"/>
-    <sheet name="Austin" sheetId="43" r:id="rId43"/>
-    <sheet name="Rogers Park" sheetId="44" r:id="rId44"/>
-    <sheet name="Mckinley Park" sheetId="45" r:id="rId45"/>
-    <sheet name="Irving Park" sheetId="46" r:id="rId46"/>
-    <sheet name="Armour Square" sheetId="47" r:id="rId47"/>
-    <sheet name="Uptown" sheetId="48" r:id="rId48"/>
-    <sheet name="West Elsdon" sheetId="49" r:id="rId49"/>
-    <sheet name="Woodlawn" sheetId="50" r:id="rId50"/>
-    <sheet name="Douglas" sheetId="51" r:id="rId51"/>
-    <sheet name="Edgewater" sheetId="52" r:id="rId52"/>
+    <sheet name="Edgewater" sheetId="41" r:id="rId41"/>
+    <sheet name="Roseland" sheetId="42" r:id="rId42"/>
+    <sheet name="Chinatown" sheetId="43" r:id="rId43"/>
+    <sheet name="Austin" sheetId="44" r:id="rId44"/>
+    <sheet name="Rogers Park" sheetId="45" r:id="rId45"/>
+    <sheet name="Mckinley Park" sheetId="46" r:id="rId46"/>
+    <sheet name="Irving Park" sheetId="47" r:id="rId47"/>
+    <sheet name="Armour Square" sheetId="48" r:id="rId48"/>
+    <sheet name="Uptown" sheetId="49" r:id="rId49"/>
+    <sheet name="West Elsdon" sheetId="50" r:id="rId50"/>
+    <sheet name="Woodlawn" sheetId="51" r:id="rId51"/>
+    <sheet name="Douglas" sheetId="52" r:id="rId52"/>
     <sheet name="Morgan Park" sheetId="53" r:id="rId53"/>
     <sheet name="Chicago Lawn" sheetId="54" r:id="rId54"/>
     <sheet name="South Deering" sheetId="55" r:id="rId55"/>
@@ -905,7 +905,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1156,7 +1156,7 @@
         <v>467</v>
       </c>
       <c r="M9">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -5064,7 +5064,7 @@
         <v>25</v>
       </c>
       <c r="M27">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -6341,7 +6341,7 @@
         <v>16</v>
       </c>
       <c r="M61">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -7116,7 +7116,7 @@
         <v>16</v>
       </c>
       <c r="M81">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -7845,7 +7845,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -10226,7 +10226,7 @@
         <v>6</v>
       </c>
       <c r="M4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -10308,7 +10308,7 @@
         <v>16</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -13519,6 +13519,283 @@
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <v>12</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>6</v>
+      </c>
+      <c r="K7">
+        <v>16</v>
+      </c>
+      <c r="L7">
+        <v>8</v>
+      </c>
+      <c r="M7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>21</v>
+      </c>
+      <c r="D8">
+        <v>21</v>
+      </c>
+      <c r="E8">
+        <v>19</v>
+      </c>
+      <c r="F8">
+        <v>19</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
+      <c r="J8">
+        <v>9</v>
+      </c>
+      <c r="K8">
+        <v>12</v>
+      </c>
+      <c r="L8">
+        <v>12</v>
+      </c>
+      <c r="M8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>24</v>
+      </c>
+      <c r="C9">
+        <v>27</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>29</v>
+      </c>
+      <c r="G9">
+        <v>18</v>
+      </c>
+      <c r="H9">
+        <v>18</v>
+      </c>
+      <c r="I9">
+        <v>23</v>
+      </c>
+      <c r="J9">
+        <v>19</v>
+      </c>
+      <c r="K9">
+        <v>34</v>
+      </c>
+      <c r="L9">
+        <v>25</v>
+      </c>
+      <c r="M9">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -13838,7 +14115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14105,324 +14382,6 @@
       </c>
       <c r="M9">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>8</v>
-      </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <v>7</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-      <c r="K3">
-        <v>12</v>
-      </c>
-      <c r="L3">
-        <v>14</v>
-      </c>
-      <c r="M3">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>23</v>
-      </c>
-      <c r="C8">
-        <v>31</v>
-      </c>
-      <c r="D8">
-        <v>22</v>
-      </c>
-      <c r="E8">
-        <v>44</v>
-      </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-      <c r="G8">
-        <v>24</v>
-      </c>
-      <c r="H8">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>34</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>24</v>
-      </c>
-      <c r="L8">
-        <v>14</v>
-      </c>
-      <c r="M8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>46</v>
-      </c>
-      <c r="C9">
-        <v>59</v>
-      </c>
-      <c r="D9">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>73</v>
-      </c>
-      <c r="F9">
-        <v>114</v>
-      </c>
-      <c r="G9">
-        <v>58</v>
-      </c>
-      <c r="H9">
-        <v>41</v>
-      </c>
-      <c r="I9">
-        <v>44</v>
-      </c>
-      <c r="J9">
-        <v>20</v>
-      </c>
-      <c r="K9">
-        <v>25</v>
-      </c>
-      <c r="L9">
-        <v>27</v>
-      </c>
-      <c r="M9">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>78</v>
-      </c>
-      <c r="C10">
-        <v>99</v>
-      </c>
-      <c r="D10">
-        <v>65</v>
-      </c>
-      <c r="E10">
-        <v>130</v>
-      </c>
-      <c r="F10">
-        <v>167</v>
-      </c>
-      <c r="G10">
-        <v>92</v>
-      </c>
-      <c r="H10">
-        <v>104</v>
-      </c>
-      <c r="I10">
-        <v>89</v>
-      </c>
-      <c r="J10">
-        <v>67</v>
-      </c>
-      <c r="K10">
-        <v>71</v>
-      </c>
-      <c r="L10">
-        <v>61</v>
-      </c>
-      <c r="M10">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -14495,73 +14454,82 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <v>3</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
         <v>8</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>5</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
       <c r="I3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -14576,23 +14544,20 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>2</v>
@@ -14602,7 +14567,7 @@
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F6">
+      <c r="K6">
         <v>1</v>
       </c>
     </row>
@@ -14610,7 +14575,7 @@
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I7">
+      <c r="L7">
         <v>1</v>
       </c>
     </row>
@@ -14619,40 +14584,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="C8">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D8">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="F8">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G8">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="J8">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="K8">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="L8">
         <v>14</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -14660,40 +14625,40 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C9">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D9">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="E9">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F9">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="G9">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="H9">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="I9">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L9">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="M9">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -14701,40 +14666,40 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C10">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="D10">
+        <v>65</v>
+      </c>
+      <c r="E10">
+        <v>130</v>
+      </c>
+      <c r="F10">
+        <v>167</v>
+      </c>
+      <c r="G10">
+        <v>92</v>
+      </c>
+      <c r="H10">
+        <v>104</v>
+      </c>
+      <c r="I10">
+        <v>89</v>
+      </c>
+      <c r="J10">
+        <v>67</v>
+      </c>
+      <c r="K10">
         <v>71</v>
       </c>
-      <c r="E10">
-        <v>101</v>
-      </c>
-      <c r="F10">
-        <v>70</v>
-      </c>
-      <c r="G10">
+      <c r="L10">
+        <v>61</v>
+      </c>
+      <c r="M10">
         <v>53</v>
-      </c>
-      <c r="H10">
-        <v>39</v>
-      </c>
-      <c r="I10">
-        <v>49</v>
-      </c>
-      <c r="J10">
-        <v>47</v>
-      </c>
-      <c r="K10">
-        <v>54</v>
-      </c>
-      <c r="L10">
-        <v>59</v>
-      </c>
-      <c r="M10">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -14744,7 +14709,7 @@
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -14808,19 +14773,31 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
       <c r="I2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -14833,136 +14810,208 @@
       <c r="C3">
         <v>1</v>
       </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
       <c r="E3">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>8</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
       <c r="K5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
         <v>6</v>
       </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
       <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>11</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>7</v>
-      </c>
-      <c r="C7">
+      <c r="F8">
+        <v>15</v>
+      </c>
+      <c r="G8">
+        <v>9</v>
+      </c>
+      <c r="H8">
+        <v>14</v>
+      </c>
+      <c r="I8">
         <v>13</v>
       </c>
-      <c r="D7">
+      <c r="J8">
+        <v>13</v>
+      </c>
+      <c r="K8">
+        <v>14</v>
+      </c>
+      <c r="L8">
+        <v>14</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>11</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
+      <c r="B9">
+        <v>56</v>
+      </c>
+      <c r="C9">
+        <v>61</v>
+      </c>
+      <c r="D9">
+        <v>54</v>
+      </c>
+      <c r="E9">
+        <v>80</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9">
+        <v>32</v>
+      </c>
+      <c r="H9">
+        <v>21</v>
+      </c>
+      <c r="I9">
+        <v>24</v>
+      </c>
+      <c r="J9">
+        <v>30</v>
+      </c>
+      <c r="K9">
+        <v>24</v>
+      </c>
+      <c r="L9">
+        <v>34</v>
+      </c>
+      <c r="M9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
+      <c r="B10">
+        <v>59</v>
+      </c>
+      <c r="C10">
+        <v>76</v>
+      </c>
+      <c r="D10">
+        <v>71</v>
+      </c>
+      <c r="E10">
+        <v>101</v>
+      </c>
+      <c r="F10">
+        <v>70</v>
+      </c>
+      <c r="G10">
+        <v>53</v>
+      </c>
+      <c r="H10">
+        <v>39</v>
+      </c>
+      <c r="I10">
+        <v>49</v>
+      </c>
+      <c r="J10">
+        <v>47</v>
+      </c>
+      <c r="K10">
+        <v>54</v>
+      </c>
+      <c r="L10">
+        <v>59</v>
+      </c>
+      <c r="M10">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -15036,31 +15085,19 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -15070,34 +15107,19 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
       <c r="H3">
         <v>1</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -15105,7 +15127,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -15117,10 +15139,10 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -15129,24 +15151,12 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -15155,40 +15165,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -15196,40 +15206,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -15306,13 +15316,16 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -15321,10 +15334,10 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -15344,38 +15357,32 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>6</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -15384,40 +15391,40 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -15425,40 +15432,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="D6">
-        <v>13</v>
-      </c>
       <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
       <c r="M6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -15466,40 +15473,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I7">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="K7">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -15508,6 +15515,276 @@
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>15</v>
+      </c>
+      <c r="K5">
+        <v>11</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>47</v>
+      </c>
+      <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>16</v>
+      </c>
+      <c r="I7">
+        <v>27</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>25</v>
+      </c>
+      <c r="L7">
+        <v>40</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15792,205 +16069,6 @@
       </c>
       <c r="M9">
         <v>17</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>12</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>9</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>12</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>3</v>
-      </c>
-      <c r="J6">
-        <v>10</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -16292,6 +16370,205 @@
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>12</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>9</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>10</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -16548,7 +16825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16795,283 +17072,6 @@
       </c>
       <c r="M8">
         <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>6</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>12</v>
-      </c>
-      <c r="I7">
-        <v>7</v>
-      </c>
-      <c r="J7">
-        <v>6</v>
-      </c>
-      <c r="K7">
-        <v>16</v>
-      </c>
-      <c r="L7">
-        <v>8</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>20</v>
-      </c>
-      <c r="C8">
-        <v>21</v>
-      </c>
-      <c r="D8">
-        <v>21</v>
-      </c>
-      <c r="E8">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>19</v>
-      </c>
-      <c r="G8">
-        <v>7</v>
-      </c>
-      <c r="H8">
-        <v>5</v>
-      </c>
-      <c r="I8">
-        <v>10</v>
-      </c>
-      <c r="J8">
-        <v>9</v>
-      </c>
-      <c r="K8">
-        <v>12</v>
-      </c>
-      <c r="L8">
-        <v>12</v>
-      </c>
-      <c r="M8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>24</v>
-      </c>
-      <c r="C9">
-        <v>27</v>
-      </c>
-      <c r="D9">
-        <v>30</v>
-      </c>
-      <c r="E9">
-        <v>25</v>
-      </c>
-      <c r="F9">
-        <v>29</v>
-      </c>
-      <c r="G9">
-        <v>18</v>
-      </c>
-      <c r="H9">
-        <v>18</v>
-      </c>
-      <c r="I9">
-        <v>23</v>
-      </c>
-      <c r="J9">
-        <v>19</v>
-      </c>
-      <c r="K9">
-        <v>34</v>
-      </c>
-      <c r="L9">
-        <v>25</v>
-      </c>
-      <c r="M9">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-12
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -1039,7 +1039,7 @@
         <v>25</v>
       </c>
       <c r="M6">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1156,7 +1156,7 @@
         <v>467</v>
       </c>
       <c r="M9">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>901</v>
+        <v>903</v>
       </c>
     </row>
   </sheetData>
@@ -1409,7 +1409,7 @@
         <v>1</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1472,7 +1472,7 @@
         <v>43</v>
       </c>
       <c r="M7">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1554,7 +1554,7 @@
         <v>102</v>
       </c>
       <c r="M9">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -5105,7 +5105,7 @@
         <v>102</v>
       </c>
       <c r="M28">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -5403,7 +5403,7 @@
         <v>98</v>
       </c>
       <c r="M36">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -5982,7 +5982,7 @@
         <v>12</v>
       </c>
       <c r="M51">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -7845,7 +7845,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>901</v>
+        <v>903</v>
       </c>
     </row>
   </sheetData>
@@ -20369,7 +20369,7 @@
         <v>2</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -20497,7 +20497,7 @@
         <v>12</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -25252,7 +25252,7 @@
         <v>13</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -25431,7 +25431,7 @@
         <v>98</v>
       </c>
       <c r="M10">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-13
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -18,14 +18,14 @@
     <sheet name="Grand Crossing" sheetId="9" r:id="rId9"/>
     <sheet name="Englewood" sheetId="10" r:id="rId10"/>
     <sheet name="Loop" sheetId="11" r:id="rId11"/>
-    <sheet name="Grand Boulevard" sheetId="12" r:id="rId12"/>
-    <sheet name="Old Town" sheetId="13" r:id="rId13"/>
-    <sheet name="Gage Park" sheetId="14" r:id="rId14"/>
-    <sheet name="Lower West Side" sheetId="15" r:id="rId15"/>
-    <sheet name="Little Italy, UIC" sheetId="16" r:id="rId16"/>
-    <sheet name="Chatham" sheetId="17" r:id="rId17"/>
-    <sheet name="Albany Park" sheetId="18" r:id="rId18"/>
-    <sheet name="Wicker Park" sheetId="19" r:id="rId19"/>
+    <sheet name="Old Town" sheetId="12" r:id="rId12"/>
+    <sheet name="Gage Park" sheetId="13" r:id="rId13"/>
+    <sheet name="Lower West Side" sheetId="14" r:id="rId14"/>
+    <sheet name="Little Italy, UIC" sheetId="15" r:id="rId15"/>
+    <sheet name="Chatham" sheetId="16" r:id="rId16"/>
+    <sheet name="Albany Park" sheetId="17" r:id="rId17"/>
+    <sheet name="Wicker Park" sheetId="18" r:id="rId18"/>
+    <sheet name="Grand Boulevard" sheetId="19" r:id="rId19"/>
     <sheet name="Belmont Cragin" sheetId="20" r:id="rId20"/>
     <sheet name="West Ridge" sheetId="21" r:id="rId21"/>
     <sheet name="Lake View" sheetId="22" r:id="rId22"/>
@@ -56,15 +56,15 @@
     <sheet name="Near South Side" sheetId="47" r:id="rId47"/>
     <sheet name="Roseland" sheetId="48" r:id="rId48"/>
     <sheet name="Auburn Gresham" sheetId="49" r:id="rId49"/>
-    <sheet name="Chinatown" sheetId="50" r:id="rId50"/>
-    <sheet name="Mckinley Park" sheetId="51" r:id="rId51"/>
-    <sheet name="Irving Park" sheetId="52" r:id="rId52"/>
-    <sheet name="Armour Square" sheetId="53" r:id="rId53"/>
-    <sheet name="Uptown" sheetId="54" r:id="rId54"/>
-    <sheet name="West Elsdon" sheetId="55" r:id="rId55"/>
-    <sheet name="Douglas" sheetId="56" r:id="rId56"/>
-    <sheet name="Morgan Park" sheetId="57" r:id="rId57"/>
-    <sheet name="Chicago Lawn" sheetId="58" r:id="rId58"/>
+    <sheet name="Chicago Lawn" sheetId="50" r:id="rId50"/>
+    <sheet name="Chinatown" sheetId="51" r:id="rId51"/>
+    <sheet name="Mckinley Park" sheetId="52" r:id="rId52"/>
+    <sheet name="Irving Park" sheetId="53" r:id="rId53"/>
+    <sheet name="Armour Square" sheetId="54" r:id="rId54"/>
+    <sheet name="Uptown" sheetId="55" r:id="rId55"/>
+    <sheet name="West Elsdon" sheetId="56" r:id="rId56"/>
+    <sheet name="Douglas" sheetId="57" r:id="rId57"/>
+    <sheet name="Morgan Park" sheetId="58" r:id="rId58"/>
     <sheet name="South Deering" sheetId="59" r:id="rId59"/>
     <sheet name="Fuller Park" sheetId="60" r:id="rId60"/>
     <sheet name="Brighton Park" sheetId="61" r:id="rId61"/>
@@ -905,7 +905,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1918,264 +1918,6 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>4</v>
-      </c>
-      <c r="M3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>6</v>
-      </c>
-      <c r="L5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>15</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
-      </c>
-      <c r="K6">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>24</v>
-      </c>
-      <c r="C7">
-        <v>29</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>16</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
-      <c r="J7">
-        <v>20</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>16</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2440,7 +2182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2717,7 +2459,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2958,7 +2700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3237,7 +2979,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3552,7 +3294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3801,7 +3543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4038,6 +3780,264 @@
       </c>
       <c r="M9">
         <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>29</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>19</v>
+      </c>
+      <c r="G7">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7">
+        <v>16</v>
+      </c>
+      <c r="M7">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4807,7 +4807,7 @@
         <v>7</v>
       </c>
       <c r="M20">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -5362,7 +5362,7 @@
         <v>16</v>
       </c>
       <c r="M35">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -16289,6 +16289,264 @@
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <v>15</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>7</v>
+      </c>
+      <c r="I7">
+        <v>13</v>
+      </c>
+      <c r="J7">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -16554,234 +16812,6 @@
       </c>
       <c r="M9">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>13</v>
-      </c>
-      <c r="D7">
-        <v>9</v>
-      </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>11</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
-        <v>10</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -16855,31 +16885,19 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -16889,34 +16907,19 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
       <c r="H3">
         <v>1</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -16924,7 +16927,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -16936,10 +16939,10 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -16948,24 +16951,12 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -16974,40 +16965,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -17015,40 +17006,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -17125,13 +17116,16 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -17140,10 +17134,10 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -17163,38 +17157,32 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>6</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -17203,40 +17191,40 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17244,40 +17232,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="D6">
-        <v>13</v>
-      </c>
       <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
       <c r="M6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -17285,40 +17273,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I7">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="K7">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -17327,6 +17315,276 @@
 </file>
 
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>15</v>
+      </c>
+      <c r="K5">
+        <v>11</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>47</v>
+      </c>
+      <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>16</v>
+      </c>
+      <c r="I7">
+        <v>27</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>25</v>
+      </c>
+      <c r="L7">
+        <v>40</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17618,7 +17876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17817,7 +18075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18071,7 +18329,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -18260,264 +18518,6 @@
       </c>
       <c r="M6">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>3</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>11</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>18</v>
-      </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>7</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>23</v>
-      </c>
-      <c r="C7">
-        <v>23</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>11</v>
-      </c>
-      <c r="F7">
-        <v>15</v>
-      </c>
-      <c r="G7">
-        <v>17</v>
-      </c>
-      <c r="H7">
-        <v>7</v>
-      </c>
-      <c r="I7">
-        <v>13</v>
-      </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-17
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -60,11 +60,11 @@
     <sheet name="Douglas" sheetId="51" r:id="rId51"/>
     <sheet name="Printers Row" sheetId="52" r:id="rId52"/>
     <sheet name="Hyde Park" sheetId="53" r:id="rId53"/>
-    <sheet name="Chinatown" sheetId="54" r:id="rId54"/>
-    <sheet name="Mckinley Park" sheetId="55" r:id="rId55"/>
-    <sheet name="Irving Park" sheetId="56" r:id="rId56"/>
-    <sheet name="Armour Square" sheetId="57" r:id="rId57"/>
-    <sheet name="Uptown" sheetId="58" r:id="rId58"/>
+    <sheet name="Uptown" sheetId="54" r:id="rId54"/>
+    <sheet name="Chinatown" sheetId="55" r:id="rId55"/>
+    <sheet name="Mckinley Park" sheetId="56" r:id="rId56"/>
+    <sheet name="Irving Park" sheetId="57" r:id="rId57"/>
+    <sheet name="Armour Square" sheetId="58" r:id="rId58"/>
     <sheet name="West Elsdon" sheetId="59" r:id="rId59"/>
     <sheet name="Morgan Park" sheetId="60" r:id="rId60"/>
     <sheet name="South Deering" sheetId="61" r:id="rId61"/>
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>920</v>
+        <v>923</v>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +1867,7 @@
         <v>95</v>
       </c>
       <c r="M9">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1908,7 +1908,7 @@
         <v>196</v>
       </c>
       <c r="M10">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -5064,7 +5064,7 @@
         <v>25</v>
       </c>
       <c r="M27">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -6064,7 +6064,7 @@
         <v>196</v>
       </c>
       <c r="M53">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -6341,7 +6341,7 @@
         <v>16</v>
       </c>
       <c r="M61">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -6587,7 +6587,7 @@
         <v>10</v>
       </c>
       <c r="M67">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -7362,7 +7362,7 @@
         <v>33</v>
       </c>
       <c r="M87">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -7845,7 +7845,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>920</v>
+        <v>923</v>
       </c>
     </row>
   </sheetData>
@@ -10506,7 +10506,7 @@
         <v>6</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -10547,7 +10547,7 @@
         <v>10</v>
       </c>
       <c r="M8">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -13745,7 +13745,7 @@
         <v>12</v>
       </c>
       <c r="M8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13786,7 +13786,7 @@
         <v>25</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -17319,68 +17319,86 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L2">
         <v>2</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4">
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -17388,15 +17406,15 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I5">
+      <c r="B5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="C6">
         <v>1</v>
       </c>
     </row>
@@ -17408,37 +17426,37 @@
         <v>5</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F7">
         <v>6</v>
       </c>
       <c r="G7">
+        <v>14</v>
+      </c>
+      <c r="H7">
+        <v>7</v>
+      </c>
+      <c r="I7">
+        <v>4</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
+        <v>11</v>
+      </c>
+      <c r="L7">
         <v>8</v>
       </c>
-      <c r="H7">
-        <v>8</v>
-      </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
-        <v>21</v>
-      </c>
-      <c r="L7">
-        <v>17</v>
-      </c>
       <c r="M7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -17446,40 +17464,40 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="D8">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E8">
+        <v>24</v>
+      </c>
+      <c r="F8">
+        <v>18</v>
+      </c>
+      <c r="G8">
+        <v>16</v>
+      </c>
+      <c r="H8">
+        <v>14</v>
+      </c>
+      <c r="I8">
+        <v>13</v>
+      </c>
+      <c r="J8">
         <v>15</v>
       </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>11</v>
-      </c>
-      <c r="J8">
+      <c r="K8">
+        <v>12</v>
+      </c>
+      <c r="L8">
+        <v>20</v>
+      </c>
+      <c r="M8">
         <v>9</v>
-      </c>
-      <c r="K8">
-        <v>7</v>
-      </c>
-      <c r="L8">
-        <v>7</v>
-      </c>
-      <c r="M8">
-        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17487,40 +17505,40 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="C9">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D9">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E9">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="F9">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G9">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="H9">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="I9">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="J9">
+        <v>31</v>
+      </c>
+      <c r="K9">
+        <v>35</v>
+      </c>
+      <c r="L9">
+        <v>33</v>
+      </c>
+      <c r="M9">
         <v>18</v>
-      </c>
-      <c r="K9">
-        <v>33</v>
-      </c>
-      <c r="L9">
-        <v>30</v>
-      </c>
-      <c r="M9">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -17530,7 +17548,7 @@
 
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -17593,13 +17611,16 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>2</v>
+      <c r="E2">
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="J2">
@@ -17608,147 +17629,190 @@
       <c r="K2">
         <v>1</v>
       </c>
-      <c r="M2">
-        <v>1</v>
+      <c r="L2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="B3">
         <v>1</v>
       </c>
       <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
       </c>
       <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
         <v>6</v>
       </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
       <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
         <v>10</v>
       </c>
-      <c r="B7">
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
+        <v>21</v>
+      </c>
+      <c r="L7">
+        <v>17</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <v>13</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>11</v>
+      </c>
+      <c r="J8">
+        <v>9</v>
+      </c>
+      <c r="K8">
         <v>7</v>
       </c>
-      <c r="C7">
-        <v>13</v>
-      </c>
-      <c r="D7">
-        <v>9</v>
-      </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>11</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
+      <c r="L8">
+        <v>7</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7">
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9">
+        <v>15</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>26</v>
+      </c>
+      <c r="G9">
+        <v>14</v>
+      </c>
+      <c r="H9">
+        <v>21</v>
+      </c>
+      <c r="I9">
+        <v>28</v>
+      </c>
+      <c r="J9">
+        <v>18</v>
+      </c>
+      <c r="K9">
+        <v>33</v>
+      </c>
+      <c r="L9">
+        <v>30</v>
+      </c>
+      <c r="M9">
         <v>7</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -17822,31 +17886,19 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -17856,34 +17908,19 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
       <c r="H3">
         <v>1</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -17891,7 +17928,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -17903,10 +17940,10 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -17915,24 +17952,12 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -17941,40 +17966,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -17982,40 +18007,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -18092,13 +18117,16 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -18107,10 +18135,10 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -18130,38 +18158,32 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>6</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -18170,40 +18192,40 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -18211,40 +18233,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="D6">
-        <v>13</v>
-      </c>
       <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
       <c r="M6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -18252,40 +18274,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I7">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="K7">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -18295,7 +18317,7 @@
 
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -18358,26 +18380,17 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -18386,198 +18399,185 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3">
         <v>6</v>
       </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>7</v>
-      </c>
-      <c r="K3">
-        <v>7</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
       <c r="M3">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>15</v>
+      </c>
+      <c r="K5">
+        <v>11</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>21</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="G7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="L7">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="M7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>30</v>
-      </c>
-      <c r="C8">
-        <v>26</v>
-      </c>
-      <c r="D8">
-        <v>15</v>
-      </c>
-      <c r="E8">
-        <v>24</v>
-      </c>
-      <c r="F8">
-        <v>18</v>
-      </c>
-      <c r="G8">
-        <v>16</v>
-      </c>
-      <c r="H8">
-        <v>14</v>
-      </c>
-      <c r="I8">
-        <v>13</v>
-      </c>
-      <c r="J8">
-        <v>15</v>
-      </c>
-      <c r="K8">
-        <v>12</v>
-      </c>
-      <c r="L8">
-        <v>20</v>
-      </c>
-      <c r="M8">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B9">
-        <v>38</v>
-      </c>
-      <c r="C9">
-        <v>41</v>
-      </c>
-      <c r="D9">
-        <v>19</v>
-      </c>
-      <c r="E9">
-        <v>36</v>
-      </c>
-      <c r="F9">
-        <v>28</v>
-      </c>
-      <c r="G9">
-        <v>38</v>
-      </c>
-      <c r="H9">
-        <v>28</v>
-      </c>
-      <c r="I9">
-        <v>23</v>
-      </c>
-      <c r="J9">
-        <v>31</v>
-      </c>
-      <c r="K9">
-        <v>35</v>
-      </c>
-      <c r="L9">
-        <v>33</v>
-      </c>
-      <c r="M9">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-18
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -946,7 +946,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1039,7 +1039,7 @@
         <v>25</v>
       </c>
       <c r="M6">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>923</v>
+        <v>925</v>
       </c>
     </row>
   </sheetData>
@@ -2828,7 +2828,7 @@
         <v>6</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2971,7 +2971,7 @@
         <v>43</v>
       </c>
       <c r="M7">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -5941,7 +5941,7 @@
         <v>43</v>
       </c>
       <c r="M50">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -6341,7 +6341,7 @@
         <v>16</v>
       </c>
       <c r="M61">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -7845,7 +7845,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>923</v>
+        <v>925</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-19
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -905,7 +905,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -946,7 +946,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>925</v>
+        <v>928</v>
       </c>
     </row>
   </sheetData>
@@ -4366,7 +4366,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4930,7 +4930,7 @@
         <v>15</v>
       </c>
       <c r="M23">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -5254,7 +5254,7 @@
         <v>71</v>
       </c>
       <c r="M32">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -7845,7 +7845,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>925</v>
+        <v>928</v>
       </c>
     </row>
   </sheetData>
@@ -10695,7 +10695,7 @@
         <v>8</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -10860,7 +10860,7 @@
         <v>71</v>
       </c>
       <c r="M9">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -14132,7 +14132,7 @@
         <v>14</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -14302,7 +14302,7 @@
         <v>61</v>
       </c>
       <c r="M10">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -16629,7 +16629,7 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -16794,7 +16794,7 @@
         <v>15</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-21
</commit_message>
<xml_diff>
--- a/output/cta-index-crime-full-year.xlsx
+++ b/output/cta-index-crime-full-year.xlsx
@@ -19,19 +19,19 @@
     <sheet name="Englewood" sheetId="10" r:id="rId10"/>
     <sheet name="Loop" sheetId="11" r:id="rId11"/>
     <sheet name="Old Town" sheetId="12" r:id="rId12"/>
-    <sheet name="Gage Park" sheetId="13" r:id="rId13"/>
-    <sheet name="Lower West Side" sheetId="14" r:id="rId14"/>
-    <sheet name="Little Italy, UIC" sheetId="15" r:id="rId15"/>
-    <sheet name="Chatham" sheetId="16" r:id="rId16"/>
-    <sheet name="Albany Park" sheetId="17" r:id="rId17"/>
-    <sheet name="Wicker Park" sheetId="18" r:id="rId18"/>
-    <sheet name="Grand Boulevard" sheetId="19" r:id="rId19"/>
-    <sheet name="Belmont Cragin" sheetId="20" r:id="rId20"/>
-    <sheet name="West Ridge" sheetId="21" r:id="rId21"/>
-    <sheet name="Lake View" sheetId="22" r:id="rId22"/>
-    <sheet name="South Shore" sheetId="23" r:id="rId23"/>
-    <sheet name="Avondale" sheetId="24" r:id="rId24"/>
-    <sheet name="Mount Greenwood" sheetId="25" r:id="rId25"/>
+    <sheet name="Lower West Side" sheetId="13" r:id="rId13"/>
+    <sheet name="Little Italy, UIC" sheetId="14" r:id="rId14"/>
+    <sheet name="Chatham" sheetId="15" r:id="rId15"/>
+    <sheet name="Albany Park" sheetId="16" r:id="rId16"/>
+    <sheet name="Wicker Park" sheetId="17" r:id="rId17"/>
+    <sheet name="Grand Boulevard" sheetId="18" r:id="rId18"/>
+    <sheet name="Belmont Cragin" sheetId="19" r:id="rId19"/>
+    <sheet name="West Ridge" sheetId="20" r:id="rId20"/>
+    <sheet name="Lake View" sheetId="21" r:id="rId21"/>
+    <sheet name="South Shore" sheetId="22" r:id="rId22"/>
+    <sheet name="Avondale" sheetId="23" r:id="rId23"/>
+    <sheet name="Mount Greenwood" sheetId="24" r:id="rId24"/>
+    <sheet name="Gage Park" sheetId="25" r:id="rId25"/>
     <sheet name="West Loop" sheetId="26" r:id="rId26"/>
     <sheet name="Rush &amp; Division" sheetId="27" r:id="rId27"/>
     <sheet name="North Lawndale" sheetId="28" r:id="rId28"/>
@@ -62,14 +62,14 @@
     <sheet name="Hyde Park" sheetId="53" r:id="rId53"/>
     <sheet name="Uptown" sheetId="54" r:id="rId54"/>
     <sheet name="Little Village" sheetId="55" r:id="rId55"/>
-    <sheet name="Chinatown" sheetId="56" r:id="rId56"/>
-    <sheet name="Mckinley Park" sheetId="57" r:id="rId57"/>
-    <sheet name="Irving Park" sheetId="58" r:id="rId58"/>
-    <sheet name="Armour Square" sheetId="59" r:id="rId59"/>
-    <sheet name="West Elsdon" sheetId="60" r:id="rId60"/>
-    <sheet name="Morgan Park" sheetId="61" r:id="rId61"/>
-    <sheet name="South Deering" sheetId="62" r:id="rId62"/>
-    <sheet name="Fuller Park" sheetId="63" r:id="rId63"/>
+    <sheet name="Fuller Park" sheetId="56" r:id="rId56"/>
+    <sheet name="Chinatown" sheetId="57" r:id="rId57"/>
+    <sheet name="Mckinley Park" sheetId="58" r:id="rId58"/>
+    <sheet name="Irving Park" sheetId="59" r:id="rId59"/>
+    <sheet name="Armour Square" sheetId="60" r:id="rId60"/>
+    <sheet name="West Elsdon" sheetId="61" r:id="rId61"/>
+    <sheet name="Morgan Park" sheetId="62" r:id="rId62"/>
+    <sheet name="South Deering" sheetId="63" r:id="rId63"/>
     <sheet name="Brighton Park" sheetId="64" r:id="rId64"/>
     <sheet name="Montclare" sheetId="65" r:id="rId65"/>
     <sheet name="Lincoln Park" sheetId="66" r:id="rId66"/>
@@ -946,7 +946,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1197,7 +1197,7 @@
         <v>703</v>
       </c>
       <c r="M10">
-        <v>418</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1238,7 +1238,7 @@
         <v>1604</v>
       </c>
       <c r="M11">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
   </sheetData>
@@ -2184,283 +2184,6 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="I7">
-        <v>3</v>
-      </c>
-      <c r="J7">
-        <v>4</v>
-      </c>
-      <c r="K7">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>5</v>
-      </c>
-      <c r="M7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>11</v>
-      </c>
-      <c r="C8">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>24</v>
-      </c>
-      <c r="E8">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>10</v>
-      </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="H8">
-        <v>4</v>
-      </c>
-      <c r="I8">
-        <v>4</v>
-      </c>
-      <c r="J8">
-        <v>4</v>
-      </c>
-      <c r="K8">
-        <v>4</v>
-      </c>
-      <c r="L8">
-        <v>3</v>
-      </c>
-      <c r="M8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>17</v>
-      </c>
-      <c r="C9">
-        <v>27</v>
-      </c>
-      <c r="D9">
-        <v>35</v>
-      </c>
-      <c r="E9">
-        <v>28</v>
-      </c>
-      <c r="F9">
-        <v>15</v>
-      </c>
-      <c r="G9">
-        <v>9</v>
-      </c>
-      <c r="H9">
-        <v>5</v>
-      </c>
-      <c r="I9">
-        <v>9</v>
-      </c>
-      <c r="J9">
-        <v>11</v>
-      </c>
-      <c r="K9">
-        <v>19</v>
-      </c>
-      <c r="L9">
-        <v>16</v>
-      </c>
-      <c r="M9">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2700,7 +2423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2828,7 +2551,7 @@
         <v>6</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2971,7 +2694,7 @@
         <v>43</v>
       </c>
       <c r="M7">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2979,7 +2702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3294,7 +3017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3543,7 +3266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3787,7 +3510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4038,6 +3761,219 @@
       </c>
       <c r="M7">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>9</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>9</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4366,7 +4302,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5064,7 +5000,7 @@
         <v>25</v>
       </c>
       <c r="M27">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -5146,7 +5082,7 @@
         <v>37</v>
       </c>
       <c r="M29">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -5616,7 +5552,7 @@
         <v>7</v>
       </c>
       <c r="M42">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -5941,7 +5877,7 @@
         <v>43</v>
       </c>
       <c r="M50">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -6979,7 +6915,7 @@
         <v>62</v>
       </c>
       <c r="M77">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -7845,7 +7781,7 @@
         <v>1604</v>
       </c>
       <c r="M99">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
   </sheetData>
@@ -7955,219 +7891,6 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>7</v>
-      </c>
-      <c r="E7">
-        <v>11</v>
-      </c>
-      <c r="F7">
-        <v>7</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <v>9</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>3</v>
-      </c>
-      <c r="M7">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -8344,7 +8067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8640,7 +8363,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8911,7 +8634,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9163,7 +8886,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9219,6 +8942,283 @@
       </c>
       <c r="D4">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <v>5</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>24</v>
+      </c>
+      <c r="E8">
+        <v>19</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>4</v>
+      </c>
+      <c r="I8">
+        <v>4</v>
+      </c>
+      <c r="J8">
+        <v>4</v>
+      </c>
+      <c r="K8">
+        <v>4</v>
+      </c>
+      <c r="L8">
+        <v>3</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>27</v>
+      </c>
+      <c r="D9">
+        <v>35</v>
+      </c>
+      <c r="E9">
+        <v>28</v>
+      </c>
+      <c r="F9">
+        <v>15</v>
+      </c>
+      <c r="G9">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>5</v>
+      </c>
+      <c r="I9">
+        <v>9</v>
+      </c>
+      <c r="J9">
+        <v>11</v>
+      </c>
+      <c r="K9">
+        <v>19</v>
+      </c>
+      <c r="L9">
+        <v>16</v>
+      </c>
+      <c r="M9">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -13748,7 +13748,7 @@
         <v>12</v>
       </c>
       <c r="M8">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13789,7 +13789,7 @@
         <v>25</v>
       </c>
       <c r="M9">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -14264,7 +14264,7 @@
         <v>27</v>
       </c>
       <c r="M9">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -14305,7 +14305,7 @@
         <v>61</v>
       </c>
       <c r="M10">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -15673,7 +15673,7 @@
         <v>25</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -15714,7 +15714,7 @@
         <v>62</v>
       </c>
       <c r="M10">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -17208,7 +17208,7 @@
         <v>3</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17249,7 +17249,7 @@
         <v>7</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -17797,7 +17797,7 @@
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -17857,26 +17857,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
+      <c r="D2">
+        <v>2</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17884,57 +17884,63 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H4">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="C5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="H6">
         <v>1</v>
       </c>
     </row>
@@ -17943,40 +17949,40 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7">
         <v>4</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G7">
         <v>8</v>
       </c>
       <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7">
+        <v>9</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
+        <v>22</v>
+      </c>
+      <c r="L7">
+        <v>22</v>
+      </c>
+      <c r="M7">
         <v>8</v>
-      </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
-        <v>21</v>
-      </c>
-      <c r="L7">
-        <v>17</v>
-      </c>
-      <c r="M7">
-        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -17984,37 +17990,37 @@
         <v>9</v>
       </c>
       <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8">
         <v>11</v>
       </c>
-      <c r="C8">
-        <v>4</v>
-      </c>
       <c r="D8">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E8">
+        <v>19</v>
+      </c>
+      <c r="F8">
         <v>15</v>
       </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
       <c r="G8">
         <v>4</v>
       </c>
       <c r="H8">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I8">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J8">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K8">
         <v>7</v>
       </c>
       <c r="L8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M8">
         <v>3</v>
@@ -18025,40 +18031,40 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D9">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="E9">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F9">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G9">
         <v>14</v>
       </c>
       <c r="H9">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="I9">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="J9">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="K9">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L9">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M9">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -18068,7 +18074,7 @@
 
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -18131,13 +18137,16 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>2</v>
+      <c r="E2">
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="J2">
@@ -18146,147 +18155,190 @@
       <c r="K2">
         <v>1</v>
       </c>
-      <c r="M2">
-        <v>1</v>
+      <c r="L2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="B3">
         <v>1</v>
       </c>
       <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
       </c>
       <c r="L3">
+        <v>4</v>
+      </c>
+      <c r="M3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
         <v>6</v>
       </c>
-      <c r="C6">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
       <c r="F6">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
         <v>10</v>
       </c>
-      <c r="B7">
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
+        <v>21</v>
+      </c>
+      <c r="L7">
+        <v>17</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <v>13</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>11</v>
+      </c>
+      <c r="J8">
+        <v>9</v>
+      </c>
+      <c r="K8">
         <v>7</v>
       </c>
-      <c r="C7">
-        <v>13</v>
-      </c>
-      <c r="D7">
-        <v>9</v>
-      </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>11</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>3</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
+      <c r="L8">
+        <v>7</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7">
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9">
+        <v>15</v>
+      </c>
+      <c r="E9">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>26</v>
+      </c>
+      <c r="G9">
+        <v>14</v>
+      </c>
+      <c r="H9">
+        <v>21</v>
+      </c>
+      <c r="I9">
+        <v>28</v>
+      </c>
+      <c r="J9">
+        <v>18</v>
+      </c>
+      <c r="K9">
+        <v>33</v>
+      </c>
+      <c r="L9">
+        <v>30</v>
+      </c>
+      <c r="M9">
         <v>7</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -18360,31 +18412,19 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -18394,34 +18434,19 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
       <c r="H3">
         <v>1</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2</v>
+      <c r="J3">
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -18429,7 +18454,7 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
@@ -18441,10 +18466,10 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -18453,24 +18478,12 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -18479,40 +18492,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -18520,40 +18533,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -18630,13 +18643,16 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -18645,10 +18661,10 @@
         <v>4</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -18668,38 +18684,32 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>6</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -18708,40 +18718,40 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -18749,40 +18759,40 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="D6">
-        <v>13</v>
-      </c>
       <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>7</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>11</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
       <c r="M6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -18790,40 +18800,40 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I7">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="J7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="K7">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="L7">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -19111,10 +19121,10 @@
 
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -19174,7 +19184,31 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
       <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -19182,125 +19216,172 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>5</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J5">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>9</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>12</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>3</v>
-      </c>
-      <c r="J6">
+      <c r="B7">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>47</v>
+      </c>
+      <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>16</v>
+      </c>
+      <c r="I7">
+        <v>27</v>
+      </c>
+      <c r="J7">
+        <v>27</v>
+      </c>
+      <c r="K7">
+        <v>25</v>
+      </c>
+      <c r="L7">
+        <v>40</v>
+      </c>
+      <c r="M7">
         <v>10</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-      <c r="L6">
-        <v>3</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -19373,16 +19454,7 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
+      <c r="L2">
         <v>1</v>
       </c>
     </row>
@@ -19390,19 +19462,13 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
         <v>1</v>
       </c>
     </row>
@@ -19410,25 +19476,28 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
       <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -19437,24 +19506,39 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>9</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -19463,40 +19547,40 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G6">
         <v>4</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -19505,6 +19589,202 @@
 </file>
 
 <file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19722,286 +20002,6 @@
       </c>
       <c r="M7">
         <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>7</v>
-      </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7">
-        <v>4</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>13</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>4</v>
-      </c>
-      <c r="I7">
-        <v>9</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
-        <v>22</v>
-      </c>
-      <c r="L7">
-        <v>22</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="C8">
-        <v>11</v>
-      </c>
-      <c r="D8">
-        <v>21</v>
-      </c>
-      <c r="E8">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>15</v>
-      </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="H8">
-        <v>3</v>
-      </c>
-      <c r="I8">
-        <v>3</v>
-      </c>
-      <c r="J8">
-        <v>12</v>
-      </c>
-      <c r="K8">
-        <v>7</v>
-      </c>
-      <c r="L8">
-        <v>9</v>
-      </c>
-      <c r="M8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>16</v>
-      </c>
-      <c r="C9">
-        <v>19</v>
-      </c>
-      <c r="D9">
-        <v>29</v>
-      </c>
-      <c r="E9">
-        <v>27</v>
-      </c>
-      <c r="F9">
-        <v>29</v>
-      </c>
-      <c r="G9">
-        <v>14</v>
-      </c>
-      <c r="H9">
-        <v>10</v>
-      </c>
-      <c r="I9">
-        <v>15</v>
-      </c>
-      <c r="J9">
-        <v>25</v>
-      </c>
-      <c r="K9">
-        <v>35</v>
-      </c>
-      <c r="L9">
-        <v>37</v>
-      </c>
-      <c r="M9">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>